<commit_message>
Update Aladdin 45-day calendar with email tests and lead-path measurement
</commit_message>
<xml_diff>
--- a/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
+++ b/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rd6cbfb527a024557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="R2eb3b82e8a6d4906"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="R9b9f428762904296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="R844034da77ac4ce9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="R57354484cd444579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rbe92ea90a1304821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="R766dbdcf981d4392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="R4103c558d90c4d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="R5808d0473d2746a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="R9c4ee1ac7a3b4526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email and Measurement" sheetId="6" r:id="Rf8e03f505b564ed0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="mm/dd/yy"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,8 +61,31 @@
       <x:color rgb="FF64707A"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF555555"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,8 +107,18 @@
         <x:fgColor rgb="FFF7F2EC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF9D1725"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9E4DD"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border>
       <x:left/>
       <x:right/>
@@ -101,11 +135,26 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -136,6 +185,36 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -581,7 +660,7 @@
         <x:v>Weekly review</x:v>
       </x:c>
       <x:c r="B27" s="6" t="str">
-        <x:v>Review saves/shares, substantive replies, clicks, calls and qualified inquiries. Use results to refine the next rolling block.</x:v>
+        <x:v>Each Sunday, review tagged article and service-page sessions, form events, phone events, qualified inquiries and booked work. Keep platform views, saves and replies as supporting signals. Review the first post-change period separately because form tracking changed on October 19.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="43" customHeight="1">
@@ -630,6 +709,38 @@
       </x:c>
       <x:c r="B34" s="6" t="str">
         <x:v>Emergency Water/Fire Restoration Triage: safety, documentation and verified next steps; operations review before publication.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" t="str">
+        <x:v>Measurement update, Oct 19</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>Use tagged links from Facebook and email to the most specific article or service page. Confirm the page has the relevant residential, commercial or emergency contact action before publishing. Track form and phone events separately; recorded events are not unique leads or verified calls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" t="str">
+        <x:v>Email test</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>Add a targeted rug-care return email after the October 29 article, then consider a second pre-guest email only after reviewing clicks, tagged visits, inquiries and unsubscribes. Check Constant Contact first to avoid duplicate sends.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>Baseline caution</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>The two October 19 reports use different one-day-shifted date windows. The October 19 tracking edits also create a measurement break. Do not treat report goal events as unique qualified leads or claim improvement from a single aggregate comparison.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>Publishing and proof</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>Keep the four Strategy Canvas paths, Aladdin voice, photo-led assets and channel-specific CTAs. Verify live permalinks, service scope, uniform colors and emergency claims before scheduling.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1424,7 +1535,7 @@
         <x:v>Real rug details; condition claims verified</x:v>
       </x:c>
       <x:c r="O17" s="6" t="str">
-        <x:v>Saves</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: saves</x:v>
       </x:c>
       <x:c r="P17" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1480,7 +1591,7 @@
         <x:v>Approved facility footage; verify actual sequence and credentials</x:v>
       </x:c>
       <x:c r="O18" s="6" t="str">
-        <x:v>Video completion</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: video completion</x:v>
       </x:c>
       <x:c r="P18" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1530,13 +1641,13 @@
         <x:v>Send a general rug question</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str">
-        <x:v>October 29 hub article</x:v>
+        <x:v>Rug cleaning page on October 28; October 29 guide only after publication</x:v>
       </x:c>
       <x:c r="N19" s="6" t="str">
         <x:v>Actual rug close-up; no unsupported diagnosis Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O19" s="6" t="str">
-        <x:v>Questions</x:v>
+        <x:v>Rug-page visits; support: questions; guide visits after publication</x:v>
       </x:c>
       <x:c r="P19" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1583,16 +1694,16 @@
         <x:v>Website + Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L20" s="6" t="str">
-        <x:v>Read the guide / request evaluation</x:v>
+        <x:v>Read the guide / discuss your rug with Aladdin</x:v>
       </x:c>
       <x:c r="M20" s="6" t="str">
-        <x:v>New article: rug evaluation guide</x:v>
+        <x:v>October 29 rug evaluation guide; publish first, then use exact permalink</x:v>
       </x:c>
       <x:c r="N20" s="6" t="str">
         <x:v>Verify exact process and credential references with Aladdin</x:v>
       </x:c>
       <x:c r="O20" s="6" t="str">
-        <x:v>Article clicks</x:v>
+        <x:v>Tagged article sessions; separate form and phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P20" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1642,13 +1753,13 @@
         <x:v>Explore the gallery / call with a question</x:v>
       </x:c>
       <x:c r="M21" s="6" t="str">
-        <x:v>Rug Gallery or current product page</x:v>
+        <x:v>Current Rug Gallery or verified product page</x:v>
       </x:c>
       <x:c r="N21" s="6" t="str">
         <x:v>Authentic product photo; recheck inventory, price, rights</x:v>
       </x:c>
       <x:c r="O21" s="6" t="str">
-        <x:v>Gallery clicks</x:v>
+        <x:v>Tagged gallery/product visits and shopping actions; support: saves</x:v>
       </x:c>
       <x:c r="P21" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1683,10 +1794,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H22" s="6" t="str">
-        <x:v>One rug-care question for the weekend</x:v>
+        <x:v>After the rug evaluation guide, what would you ask next?</x:v>
       </x:c>
       <x:c r="I22" s="6" t="str">
-        <x:v>A light question about a rug detail readers want explained. Avoid forced Halloween copy.</x:v>
+        <x:v>Follow the October 29 guide with a specific question about material, dye, condition or prior repair. Answer one concern from the article, then invite readers to the full guide. Facebook links to the exact live permalink; Instagram keeps the phone CTA.</x:v>
       </x:c>
       <x:c r="J22" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -1695,16 +1806,16 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L22" s="6" t="str">
-        <x:v>Reply with a question</x:v>
+        <x:v>Read the rug evaluation guide / ask about your rug</x:v>
       </x:c>
       <x:c r="M22" s="6" t="str">
-        <x:v>Rug care series</x:v>
+        <x:v>October 29 rug evaluation guide, exact permalink after publication</x:v>
       </x:c>
       <x:c r="N22" s="6" t="str">
-        <x:v>Actual rug detail photo Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
+        <x:v>Real rug detail photo; confirm guide is live and the specific link works before scheduling</x:v>
       </x:c>
       <x:c r="O22" s="6" t="str">
-        <x:v>Replies</x:v>
+        <x:v>Tagged guide visits and form/phone events; support: replies</x:v>
       </x:c>
       <x:c r="P22" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1742,7 +1853,7 @@
         <x:v>Listen and update FAQ</x:v>
       </x:c>
       <x:c r="I23" s="6" t="str">
-        <x:v>No feed post. Review rug questions and note ideas for the next article.</x:v>
+        <x:v>No feed post. Review the preceding week: tagged website visits, form and phone events separately, qualified inquiries, booked work where available, and what questions need a clearer answer. Keep test leads out of results.</x:v>
       </x:c>
       <x:c r="J23" s="6" t="str">
         <x:v>Community management</x:v>
@@ -1760,7 +1871,7 @@
         <x:v>No new asset</x:v>
       </x:c>
       <x:c r="O23" s="6" t="str">
-        <x:v>Questions / inquiries</x:v>
+        <x:v>Tagged visits; form/phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P23" s="15" t="str">
         <x:v>Listen</x:v>
@@ -1816,7 +1927,7 @@
         <x:v>Real textile photos; avoid stain-removal guarantees</x:v>
       </x:c>
       <x:c r="O24" s="6" t="str">
-        <x:v>Saves</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: saves</x:v>
       </x:c>
       <x:c r="P24" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1872,7 +1983,7 @@
         <x:v>Approved technician footage; uniform and process check</x:v>
       </x:c>
       <x:c r="O25" s="6" t="str">
-        <x:v>Video completion</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: video completion</x:v>
       </x:c>
       <x:c r="P25" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1922,13 +2033,13 @@
         <x:v>Vote</x:v>
       </x:c>
       <x:c r="M26" s="6" t="str">
-        <x:v>November 5 hub article</x:v>
+        <x:v>Upholstery page on November 4; November 5 guide only after publication</x:v>
       </x:c>
       <x:c r="N26" s="6" t="str">
         <x:v>Four real surface photos; no icon-only card Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O26" s="6" t="str">
-        <x:v>Votes</x:v>
+        <x:v>Upholstery-page visits; support: votes; guide visits after publication</x:v>
       </x:c>
       <x:c r="P26" s="6" t="str">
         <x:v>Planned</x:v>
@@ -1975,16 +2086,16 @@
         <x:v>Website + Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L27" s="6" t="str">
-        <x:v>Read the guide / request assessment</x:v>
+        <x:v>Read the guide / request residential care</x:v>
       </x:c>
       <x:c r="M27" s="6" t="str">
-        <x:v>New article: upholstery care conversation</x:v>
+        <x:v>November 5 upholstery guide; publish first, then use exact permalink</x:v>
       </x:c>
       <x:c r="N27" s="6" t="str">
         <x:v>Verify fabric-care claims and live permalink</x:v>
       </x:c>
       <x:c r="O27" s="6" t="str">
-        <x:v>Article clicks</x:v>
+        <x:v>Tagged article sessions; separate form and phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P27" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2040,7 +2151,7 @@
         <x:v>Customer permission if identifiable; actual team photo</x:v>
       </x:c>
       <x:c r="O28" s="6" t="str">
-        <x:v>Meaningful comments</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: meaningful comments</x:v>
       </x:c>
       <x:c r="P28" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2096,7 +2207,7 @@
         <x:v>Real furniture detail photo Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O29" s="6" t="str">
-        <x:v>Replies</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: replies</x:v>
       </x:c>
       <x:c r="P29" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2134,7 +2245,7 @@
         <x:v>Listen and log needs</x:v>
       </x:c>
       <x:c r="I30" s="6" t="str">
-        <x:v>No feed post. Record recurring fabric and floor questions for next planning cycle.</x:v>
+        <x:v>No feed post. Review the preceding week: tagged website visits, form and phone events separately, qualified inquiries, booked work where available, and what questions need a clearer answer. Keep test leads out of results.</x:v>
       </x:c>
       <x:c r="J30" s="6" t="str">
         <x:v>Community management</x:v>
@@ -2152,7 +2263,7 @@
         <x:v>No new asset</x:v>
       </x:c>
       <x:c r="O30" s="6" t="str">
-        <x:v>Questions</x:v>
+        <x:v>Tagged visits; form/phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P30" s="15" t="str">
         <x:v>Listen</x:v>
@@ -2208,7 +2319,7 @@
         <x:v>Verify safety language and confirmed contact path with restoration operations</x:v>
       </x:c>
       <x:c r="O31" s="6" t="str">
-        <x:v>Saves</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: saves</x:v>
       </x:c>
       <x:c r="P31" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2264,7 +2375,7 @@
         <x:v>No customer records or private site details; operations review required</x:v>
       </x:c>
       <x:c r="O32" s="6" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: shares</x:v>
       </x:c>
       <x:c r="P32" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2299,10 +2410,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H33" s="6" t="str">
-        <x:v>What would you want explained first?</x:v>
+        <x:v>What should you document after water enters a room?</x:v>
       </x:c>
       <x:c r="I33" s="6" t="str">
-        <x:v>Ask whether safety, documentation, response steps or timing needs the clearest explanation. Invite general questions, not a diagnosis in comments.</x:v>
+        <x:v>Use one practical, operations-approved documentation question as the lead-in to the November 12 guide. Refer an active water or fire issue to the confirmed emergency phone path; do not imply a public comment is triage.</x:v>
       </x:c>
       <x:c r="J33" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2311,16 +2422,16 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L33" s="6" t="str">
-        <x:v>Reply or call for an active issue</x:v>
+        <x:v>Read current restoration guidance / call for active help</x:v>
       </x:c>
       <x:c r="M33" s="6" t="str">
-        <x:v>November 12 hub article</x:v>
+        <x:v>Water-damage restoration page on November 11; November 12 guide only after publication</x:v>
       </x:c>
       <x:c r="N33" s="6" t="str">
-        <x:v>Caption must remain visible; no unverified response-time promise</x:v>
+        <x:v>Operations and compliance approval of safety and response language; verify emergency number and live permalink</x:v>
       </x:c>
       <x:c r="O33" s="6" t="str">
-        <x:v>Replies</x:v>
+        <x:v>Tagged restoration-page visits and phone events; support: questions</x:v>
       </x:c>
       <x:c r="P33" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2370,13 +2481,13 @@
         <x:v>Read the guide / call for active help</x:v>
       </x:c>
       <x:c r="M34" s="6" t="str">
-        <x:v>New article: water-damage first conversation</x:v>
+        <x:v>November 12 water-damage guide; publish first, then use exact permalink</x:v>
       </x:c>
       <x:c r="N34" s="6" t="str">
         <x:v>Restoration operations and compliance review; verified phone and live permalink before social</x:v>
       </x:c>
       <x:c r="O34" s="6" t="str">
-        <x:v>Article clicks</x:v>
+        <x:v>Tagged article sessions; separate form and phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P34" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2432,7 +2543,7 @@
         <x:v>Employee permission; verified role; correct uniform; no invented response claim</x:v>
       </x:c>
       <x:c r="O35" s="6" t="str">
-        <x:v>Meaningful comments</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: meaningful comments</x:v>
       </x:c>
       <x:c r="P35" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2488,7 +2599,7 @@
         <x:v>No guarantee of availability or response time</x:v>
       </x:c>
       <x:c r="O36" s="6" t="str">
-        <x:v>Replies</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: replies</x:v>
       </x:c>
       <x:c r="P36" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2526,7 +2637,7 @@
         <x:v>Listen and review readiness questions</x:v>
       </x:c>
       <x:c r="I37" s="6" t="str">
-        <x:v>No feed post. Record where the guide or triage language remains unclear.</x:v>
+        <x:v>No feed post. Review the preceding week: tagged website visits, form and phone events separately, qualified inquiries, booked work where available, and what questions need a clearer answer. Keep test leads out of results.</x:v>
       </x:c>
       <x:c r="J37" s="6" t="str">
         <x:v>Community management</x:v>
@@ -2544,7 +2655,7 @@
         <x:v>No new asset</x:v>
       </x:c>
       <x:c r="O37" s="6" t="str">
-        <x:v>Questions / clicks</x:v>
+        <x:v>Tagged visits; form/phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P37" s="15" t="str">
         <x:v>Listen</x:v>
@@ -2600,7 +2711,7 @@
         <x:v>Warm real home photos; no staged client claim</x:v>
       </x:c>
       <x:c r="O38" s="6" t="str">
-        <x:v>Saves</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: saves</x:v>
       </x:c>
       <x:c r="P38" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2656,7 +2767,7 @@
         <x:v>Real service-prep footage; verify site guidance</x:v>
       </x:c>
       <x:c r="O39" s="6" t="str">
-        <x:v>Video completion</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: video completion</x:v>
       </x:c>
       <x:c r="P39" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2706,13 +2817,13 @@
         <x:v>Vote</x:v>
       </x:c>
       <x:c r="M40" s="6" t="str">
-        <x:v>November 19 hub article</x:v>
+        <x:v>Residential services page on November 18; November 19 guide only after publication</x:v>
       </x:c>
       <x:c r="N40" s="6" t="str">
         <x:v>Real room photos; no icon-only card Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O40" s="6" t="str">
-        <x:v>Votes</x:v>
+        <x:v>Residential-page visits; support: votes; guide visits after publication</x:v>
       </x:c>
       <x:c r="P40" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2759,16 +2870,16 @@
         <x:v>Website + Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L41" s="6" t="str">
-        <x:v>Read the plan / request guidance</x:v>
+        <x:v>Read the plan / request residential care</x:v>
       </x:c>
       <x:c r="M41" s="6" t="str">
-        <x:v>New article: pre-guest care plan</x:v>
+        <x:v>November 19 pre-guest guide; publish first, then use exact permalink</x:v>
       </x:c>
       <x:c r="N41" s="6" t="str">
         <x:v>Verify scheduling language and live permalink</x:v>
       </x:c>
       <x:c r="O41" s="6" t="str">
-        <x:v>Article clicks</x:v>
+        <x:v>Tagged article sessions; separate form and phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P41" s="15" t="str">
         <x:v>Planned</x:v>
@@ -2824,7 +2935,7 @@
         <x:v>Permission and claim check; no invented review</x:v>
       </x:c>
       <x:c r="O42" s="6" t="str">
-        <x:v>Meaningful comments</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: meaningful comments</x:v>
       </x:c>
       <x:c r="P42" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2880,7 +2991,7 @@
         <x:v>Warm photo-led Story Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O43" s="6" t="str">
-        <x:v>Replies</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: replies</x:v>
       </x:c>
       <x:c r="P43" s="6" t="str">
         <x:v>Planned</x:v>
@@ -2918,7 +3029,7 @@
         <x:v>Listen before the holiday week</x:v>
       </x:c>
       <x:c r="I44" s="6" t="str">
-        <x:v>No feed post. Route time-sensitive inquiries to confirmed contact path.</x:v>
+        <x:v>No feed post. Review the preceding week: tagged website visits, form and phone events separately, qualified inquiries, booked work where available, and what questions need a clearer answer. Keep test leads out of results.</x:v>
       </x:c>
       <x:c r="J44" s="6" t="str">
         <x:v>Community management</x:v>
@@ -2936,7 +3047,7 @@
         <x:v>No new asset</x:v>
       </x:c>
       <x:c r="O44" s="6" t="str">
-        <x:v>Response quality</x:v>
+        <x:v>Tagged visits; form/phone events; qualified inquiries</x:v>
       </x:c>
       <x:c r="P44" s="6" t="str">
         <x:v>Listen</x:v>
@@ -2992,7 +3103,7 @@
         <x:v>Actual commercial setting; no private site detail</x:v>
       </x:c>
       <x:c r="O45" s="6" t="str">
-        <x:v>Shares</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: shares</x:v>
       </x:c>
       <x:c r="P45" s="6" t="str">
         <x:v>Planned</x:v>
@@ -3048,7 +3159,7 @@
         <x:v>Real facility/process footage; verify service scope and capacity</x:v>
       </x:c>
       <x:c r="O46" s="6" t="str">
-        <x:v>Video completion</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: video completion</x:v>
       </x:c>
       <x:c r="P46" s="6" t="str">
         <x:v>Planned</x:v>
@@ -3216,7 +3327,7 @@
         <x:v>Real rug/towel photo; recheck guide link and no outcome claims</x:v>
       </x:c>
       <x:c r="O49" s="6" t="str">
-        <x:v>Guide clicks</x:v>
+        <x:v>Tagged page sessions and qualified inquiries; support: guide clicks</x:v>
       </x:c>
       <x:c r="P49" s="15" t="str">
         <x:v>Planned</x:v>
@@ -3254,7 +3365,7 @@
         <x:v>What should we explain in December?</x:v>
       </x:c>
       <x:c r="I50" s="6" t="str">
-        <x:v>Story poll on rug care, fabric care, surface planning and service expectations. Feed answers into the next rolling calendar.</x:v>
+        <x:v>Ask what customers need explained in December. Use response themes together with tagged article visits, form/phone events, qualified inquiries and the email test results to shape the next calendar.</x:v>
       </x:c>
       <x:c r="J50" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -3272,7 +3383,7 @@
         <x:v>Photo-led Story, not icon card Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
       </x:c>
       <x:c r="O50" s="6" t="str">
-        <x:v>Topic votes</x:v>
+        <x:v>Topic votes and useful replies; December planning input</x:v>
       </x:c>
       <x:c r="P50" s="6" t="str">
         <x:v>Planned</x:v>
@@ -3728,13 +3839,13 @@
         <x:v>Real rug details and approved facility process</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>Assessment cues → intake Reel → rug Q&amp;A → hub → gallery</x:v>
+        <x:v>Assessment cues → intake Reel → rug Q&amp;A → Oct 29 hub → Oct 31 guide follow-up; a targeted email returns readers to the guide. Keep the Oct 30 gallery feature distinct from the care path.</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str">
-        <x:v>Save → question → evaluation</x:v>
+        <x:v>Save → ask → read guide → discuss a specific rug concern</x:v>
       </x:c>
       <x:c r="I7" s="6" t="str">
-        <x:v>Check process, inventory and product details</x:v>
+        <x:v>Publish guide before links; check existing email schedule; use a person-plus-company sender and plain text; track unsubscribes as well as inquiries.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="92" customHeight="1">
@@ -3786,13 +3897,13 @@
         <x:v>Real, approved restoration or documentation imagery</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
-        <x:v>Safe first steps → record basics → question → hub → team proof → facility contacts</x:v>
+        <x:v>Operations-approved first steps and documentation question → Nov 12 guide → relevant call path for an active issue.</x:v>
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>Save → read → call for active help</x:v>
       </x:c>
       <x:c r="I9" s="6" t="str">
-        <x:v>Restoration operations and compliance must approve safety, scope, response and insurance language</x:v>
+        <x:v>Restoration operations and compliance approve safety, scope, response and insurance language; confirm the phone path and live permalink.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="92" customHeight="1">
@@ -3815,13 +3926,13 @@
         <x:v>Real rooms and realistic appointment preparation</x:v>
       </x:c>
       <x:c r="G10" s="6" t="str">
-        <x:v>Priorities → prep Reel → room poll → hub → communication proof</x:v>
+        <x:v>Priorities → prep Reel → room poll → Nov 19 hub → communication proof; optional return email only after first email test review.</x:v>
       </x:c>
       <x:c r="H10" s="6" t="str">
         <x:v>Save → ask → plan</x:v>
       </x:c>
       <x:c r="I10" s="6" t="str">
-        <x:v>Check scheduling availability; no urgency pressure</x:v>
+        <x:v>Check scheduling availability, email fatigue and existing Constant Contact sends; no urgency pressure.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="92" customHeight="1">
@@ -4068,7 +4179,300 @@
         <x:v>Calendar calculation; verify Aladdin hours before publication</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Pro Analytics Review, Oct 19</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>Goal handoff, social-to-hub sequencing and email return path</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Test matched hooks and destinations; distinguish platform attention, website visits, form events, phone events and qualified leads.</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Report period Sep 18–Oct 17 differs from the performance PDF by one day; do not merge their baselines.</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Aladdin-Cleaning-Restoration_Pro-Analytics-Review_2026-10-19_10-58-37_CT.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Message Magnet Performance, Oct 19</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>Recorded outcomes, audience return and email response</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Form events fell while phone events rose; returning users fell; email clicks and unsubscribes both rose. Test path quality and email relevance.</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Goal events are actions, not unique leads; opens/clicks may include automation; service-area filtering is off.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Aladdin-Cleaning-Restoration_Message-Magnet-Performance_2026-10-19_11-09-46_CT.pdf</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="55" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="17" t="str">
+        <x:v>Email return tests and measurement plan</x:v>
+      </x:c>
+      <x:c r="B2" s="17"/>
+      <x:c r="C2" s="17"/>
+      <x:c r="D2" s="17"/>
+      <x:c r="E2" s="17"/>
+      <x:c r="F2" s="17"/>
+      <x:c r="G2" s="17"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="18" t="str">
+        <x:v>Calendar companion | October 19 to November 28, 2026</x:v>
+      </x:c>
+      <x:c r="B3" s="18"/>
+      <x:c r="C3" s="18"/>
+      <x:c r="D3" s="18"/>
+      <x:c r="E3" s="18"/>
+      <x:c r="F3" s="18"/>
+      <x:c r="G3" s="18"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="28" t="str">
+        <x:v>Target date</x:v>
+      </x:c>
+      <x:c r="B5" s="28" t="str">
+        <x:v>Assignment</x:v>
+      </x:c>
+      <x:c r="C5" s="28" t="str">
+        <x:v>Audience and send gate</x:v>
+      </x:c>
+      <x:c r="D5" s="28" t="str">
+        <x:v>Hub destination</x:v>
+      </x:c>
+      <x:c r="E5" s="28" t="str">
+        <x:v>Creative and next action</x:v>
+      </x:c>
+      <x:c r="F5" s="28" t="str">
+        <x:v>Measurement</x:v>
+      </x:c>
+      <x:c r="G5" s="28" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="112" customHeight="1">
+      <x:c r="A6" s="29" t="str">
+        <x:v>Oct 30</x:v>
+      </x:c>
+      <x:c r="B6" s="29" t="str">
+        <x:v>Rug care return email</x:v>
+      </x:c>
+      <x:c r="C6" s="29" t="str">
+        <x:v>Relevant existing customers or subscribers, if a suitable segment exists. Check Constant Contact schedule and suppress duplicates before sending.</x:v>
+      </x:c>
+      <x:c r="D6" s="29" t="str">
+        <x:v>October 29 Oriental rug evaluation guide, exact live permalink</x:v>
+      </x:c>
+      <x:c r="E6" s="29" t="str">
+        <x:v>Use a recognizable person + Aladdin sender, a specific subject and conversational plain text with no logo/header. Answer one rug-care question; link to the guide and its verified contact action.</x:v>
+      </x:c>
+      <x:c r="F6" s="29" t="str">
+        <x:v>Delivered, unsubscribes, clicks, tagged article sessions, separate form/phone events and qualified inquiries. Do not equate clicks with visits.</x:v>
+      </x:c>
+      <x:c r="G6" s="29" t="str">
+        <x:v>Planned test; send date and audience require schedule review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="112" customHeight="1">
+      <x:c r="A7" s="29" t="str">
+        <x:v>Nov 20</x:v>
+      </x:c>
+      <x:c r="B7" s="29" t="str">
+        <x:v>Pre-guest care return email</x:v>
+      </x:c>
+      <x:c r="C7" s="29" t="str">
+        <x:v>Conditional: review first email relevance, clicks, tagged visits, inquiries and unsubscribes; check existing sends and availability before proceeding.</x:v>
+      </x:c>
+      <x:c r="D7" s="29" t="str">
+        <x:v>November 19 practical pre-guest care guide, exact live permalink</x:v>
+      </x:c>
+      <x:c r="E7" s="29" t="str">
+        <x:v>Use the same person + company, specific subject and plain-text approach. Offer a useful planning answer without holiday urgency or unverified availability.</x:v>
+      </x:c>
+      <x:c r="F7" s="29" t="str">
+        <x:v>Delivered, unsubscribes, clicks, tagged guide sessions, separate form/phone events and qualified inquiries.</x:v>
+      </x:c>
+      <x:c r="G7" s="29" t="str">
+        <x:v>Conditional planned test</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="26"/>
+      <x:c r="B8" s="26"/>
+      <x:c r="C8" s="26"/>
+      <x:c r="D8" s="26"/>
+      <x:c r="E8" s="26"/>
+      <x:c r="F8" s="26"/>
+      <x:c r="G8" s="26"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="27" t="str">
+        <x:v>Weekly measurement and publishing checks</x:v>
+      </x:c>
+      <x:c r="B9" s="27"/>
+      <x:c r="C9" s="27"/>
+      <x:c r="D9" s="27"/>
+      <x:c r="E9" s="27"/>
+      <x:c r="F9" s="27"/>
+      <x:c r="G9" s="27"/>
+    </x:row>
+    <x:row r="10" ht="46" customHeight="1">
+      <x:c r="A10" s="28" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="str">
+        <x:v>Record separately</x:v>
+      </x:c>
+      <x:c r="C10" s="28" t="str">
+        <x:v>Decision rule</x:v>
+      </x:c>
+      <x:c r="D10" s="26"/>
+      <x:c r="E10" s="26"/>
+      <x:c r="F10" s="26"/>
+      <x:c r="G10" s="26"/>
+    </x:row>
+    <x:row r="11" ht="46" customHeight="1">
+      <x:c r="A11" s="29" t="str">
+        <x:v>Link path</x:v>
+      </x:c>
+      <x:c r="B11" s="29" t="str">
+        <x:v>Post/email ID, tagged URL, article or service landing page, CTA and final contact path</x:v>
+      </x:c>
+      <x:c r="C11" s="29" t="str">
+        <x:v>Facebook links to the exact matching Aladdin page; email links to the hub; Instagram caption uses 210-361-3930, without a raw URL.</x:v>
+      </x:c>
+      <x:c r="D11" s="26"/>
+      <x:c r="E11" s="26"/>
+      <x:c r="F11" s="26"/>
+      <x:c r="G11" s="26"/>
+    </x:row>
+    <x:row r="12" ht="46" customHeight="1">
+      <x:c r="A12" s="29" t="str">
+        <x:v>Website response</x:v>
+      </x:c>
+      <x:c r="B12" s="29" t="str">
+        <x:v>Tagged sessions to each hub and contact path; form events; phone events</x:v>
+      </x:c>
+      <x:c r="C12" s="29" t="str">
+        <x:v>Verify event definitions after the Oct 19 tracking changes. Count forms and phone actions separately; inspect source and service fit.</x:v>
+      </x:c>
+      <x:c r="D12" s="26"/>
+      <x:c r="E12" s="26"/>
+      <x:c r="F12" s="26"/>
+      <x:c r="G12" s="26"/>
+    </x:row>
+    <x:row r="13" ht="46" customHeight="1">
+      <x:c r="A13" s="29" t="str">
+        <x:v>Lead quality</x:v>
+      </x:c>
+      <x:c r="B13" s="29" t="str">
+        <x:v>Real submissions, qualified inquiries, estimates and booked work when available</x:v>
+      </x:c>
+      <x:c r="C13" s="29" t="str">
+        <x:v>Exclude marked tests; do not treat GA4 events or phone taps as unique customers or completed calls.</x:v>
+      </x:c>
+      <x:c r="D13" s="26"/>
+      <x:c r="E13" s="26"/>
+      <x:c r="F13" s="26"/>
+      <x:c r="G13" s="26"/>
+    </x:row>
+    <x:row r="14" ht="46" customHeight="1">
+      <x:c r="A14" s="29" t="str">
+        <x:v>Email response</x:v>
+      </x:c>
+      <x:c r="B14" s="29" t="str">
+        <x:v>Delivered, clicks, tagged return sessions, inquiries and unsubscribes</x:v>
+      </x:c>
+      <x:c r="C14" s="29" t="str">
+        <x:v>Clicks rose in the report, but unsubscribes rose too. Review the first send before a second or any increase in frequency.</x:v>
+      </x:c>
+      <x:c r="D14" s="26"/>
+      <x:c r="E14" s="26"/>
+      <x:c r="F14" s="26"/>
+      <x:c r="G14" s="26"/>
+    </x:row>
+    <x:row r="15" ht="46" customHeight="1">
+      <x:c r="A15" s="29" t="str">
+        <x:v>Comparison</x:v>
+      </x:c>
+      <x:c r="B15" s="29" t="str">
+        <x:v>Matched publication age, format, exposure, source and post-change reporting period</x:v>
+      </x:c>
+      <x:c r="C15" s="29" t="str">
+        <x:v>The two PDFs use different dates, and measurement changed Oct 19. Do not claim uplift from one blended baseline.</x:v>
+      </x:c>
+      <x:c r="D15" s="26"/>
+      <x:c r="E15" s="26"/>
+      <x:c r="F15" s="26"/>
+      <x:c r="G15" s="26"/>
+    </x:row>
+    <x:row r="16" ht="46" customHeight="1">
+      <x:c r="A16" s="29" t="str">
+        <x:v>Service fit</x:v>
+      </x:c>
+      <x:c r="B16" s="29" t="str">
+        <x:v>Relevant service area and actual customer problem when available</x:v>
+      </x:c>
+      <x:c r="C16" s="29" t="str">
+        <x:v>Geography is approximate and filtering is off; do not assume every session is a local prospect or a bot.</x:v>
+      </x:c>
+      <x:c r="D16" s="26"/>
+      <x:c r="E16" s="26"/>
+      <x:c r="F16" s="26"/>
+      <x:c r="G16" s="26"/>
+    </x:row>
+    <x:row r="17" ht="46" customHeight="1">
+      <x:c r="A17" s="29" t="str">
+        <x:v>Publishing gate</x:v>
+      </x:c>
+      <x:c r="B17" s="29" t="str">
+        <x:v>Live permalink, service-specific CTA, responsive contact action, image and claims approval</x:v>
+      </x:c>
+      <x:c r="C17" s="29" t="str">
+        <x:v>Use the current Strategy Canvas and voice; obtain operations approval for emergency/insurance claims and named assessment offers.</x:v>
+      </x:c>
+      <x:c r="D17" s="26"/>
+      <x:c r="E17" s="26"/>
+      <x:c r="F17" s="26"/>
+      <x:c r="G17" s="26"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A9:G9"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve layout of Aladdin calendar update notes
</commit_message>
<xml_diff>
--- a/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
+++ b/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rbe92ea90a1304821"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="R766dbdcf981d4392"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="R4103c558d90c4d97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="R5808d0473d2746a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="R9c4ee1ac7a3b4526"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email and Measurement" sheetId="6" r:id="Rf8e03f505b564ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rb5873ca60583419b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="R52bce0fce8d44093"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="R8f41fb63186041b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="Re24811e01c9143fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="R78e1a5a8047e43bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email and Measurement" sheetId="6" r:id="R0d4dab93e5894815"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="mm/dd/yy"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,6 +60,12 @@
       <x:sz val="10"/>
       <x:color rgb="FF64707A"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF8C1730"/>
+      <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
@@ -154,7 +160,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="30">
+  <x:cellXfs count="31">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -187,31 +193,34 @@
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -711,35 +720,35 @@
         <x:v>Emergency Water/Fire Restoration Triage: safety, documentation and verified next steps; operations review before publication.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35">
-      <x:c r="A35" t="str">
+    <x:row r="35" ht="62" customHeight="1">
+      <x:c r="A35" s="18" t="str">
         <x:v>Measurement update, Oct 19</x:v>
       </x:c>
-      <x:c r="B35" t="str">
+      <x:c r="B35" s="17" t="str">
         <x:v>Use tagged links from Facebook and email to the most specific article or service page. Confirm the page has the relevant residential, commercial or emergency contact action before publishing. Track form and phone events separately; recorded events are not unique leads or verified calls.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" t="str">
+    <x:row r="36" ht="62" customHeight="1">
+      <x:c r="A36" s="18" t="str">
         <x:v>Email test</x:v>
       </x:c>
-      <x:c r="B36" t="str">
+      <x:c r="B36" s="17" t="str">
         <x:v>Add a targeted rug-care return email after the October 29 article, then consider a second pre-guest email only after reviewing clicks, tagged visits, inquiries and unsubscribes. Check Constant Contact first to avoid duplicate sends.</x:v>
       </x:c>
     </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
+    <x:row r="37" ht="62" customHeight="1">
+      <x:c r="A37" s="18" t="str">
         <x:v>Baseline caution</x:v>
       </x:c>
-      <x:c r="B37" t="str">
+      <x:c r="B37" s="17" t="str">
         <x:v>The two October 19 reports use different one-day-shifted date windows. The October 19 tracking edits also create a measurement break. Do not treat report goal events as unique qualified leads or claim improvement from a single aggregate comparison.</x:v>
       </x:c>
     </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+    <x:row r="38" ht="62" customHeight="1">
+      <x:c r="A38" s="18" t="str">
         <x:v>Publishing and proof</x:v>
       </x:c>
-      <x:c r="B38" t="str">
+      <x:c r="B38" s="17" t="str">
         <x:v>Keep the four Strategy Canvas paths, Aladdin voice, photo-led assets and channel-specific CTAs. Verify live permalinks, service scope, uniform colors and emergency claims before scheduling.</x:v>
       </x:c>
     </x:row>
@@ -4179,43 +4188,43 @@
         <x:v>Calendar calculation; verify Aladdin hours before publication</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="13" ht="92" customHeight="1">
+      <x:c r="A13" s="17" t="str">
         <x:v>Pro Analytics Review, Oct 19</x:v>
       </x:c>
-      <x:c r="B13" t="str">
+      <x:c r="B13" s="17" t="str">
         <x:v>Goal handoff, social-to-hub sequencing and email return path</x:v>
       </x:c>
-      <x:c r="C13" t="str">
+      <x:c r="C13" s="17" t="str">
         <x:v>Test matched hooks and destinations; distinguish platform attention, website visits, form events, phone events and qualified leads.</x:v>
       </x:c>
-      <x:c r="D13" t="str">
+      <x:c r="D13" s="17" t="str">
         <x:v>Report period Sep 18–Oct 17 differs from the performance PDF by one day; do not merge their baselines.</x:v>
       </x:c>
-      <x:c r="E13" t="str">
+      <x:c r="E13" s="17" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F13" t="str">
+      <x:c r="F13" s="17" t="str">
         <x:v>Aladdin-Cleaning-Restoration_Pro-Analytics-Review_2026-10-19_10-58-37_CT.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
+    <x:row r="14" ht="92" customHeight="1">
+      <x:c r="A14" s="17" t="str">
         <x:v>Message Magnet Performance, Oct 19</x:v>
       </x:c>
-      <x:c r="B14" t="str">
+      <x:c r="B14" s="17" t="str">
         <x:v>Recorded outcomes, audience return and email response</x:v>
       </x:c>
-      <x:c r="C14" t="str">
+      <x:c r="C14" s="17" t="str">
         <x:v>Form events fell while phone events rose; returning users fell; email clicks and unsubscribes both rose. Test path quality and email relevance.</x:v>
       </x:c>
-      <x:c r="D14" t="str">
+      <x:c r="D14" s="17" t="str">
         <x:v>Goal events are actions, not unique leads; opens/clicks may include automation; service-area filtering is off.</x:v>
       </x:c>
-      <x:c r="E14" t="str">
+      <x:c r="E14" s="17" t="str">
         <x:v>Evidence</x:v>
       </x:c>
-      <x:c r="F14" t="str">
+      <x:c r="F14" s="17" t="str">
         <x:v>Aladdin-Cleaning-Restoration_Message-Magnet-Performance_2026-10-19_11-09-46_CT.pdf</x:v>
       </x:c>
     </x:row>
@@ -4238,235 +4247,235 @@
   </x:cols>
   <x:sheetData>
     <x:row r="2">
-      <x:c r="A2" s="17" t="str">
+      <x:c r="A2" s="20" t="str">
         <x:v>Email return tests and measurement plan</x:v>
       </x:c>
-      <x:c r="B2" s="17"/>
-      <x:c r="C2" s="17"/>
-      <x:c r="D2" s="17"/>
-      <x:c r="E2" s="17"/>
-      <x:c r="F2" s="17"/>
-      <x:c r="G2" s="17"/>
+      <x:c r="B2" s="20"/>
+      <x:c r="C2" s="20"/>
+      <x:c r="D2" s="20"/>
+      <x:c r="E2" s="20"/>
+      <x:c r="F2" s="20"/>
+      <x:c r="G2" s="20"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="18" t="str">
+      <x:c r="A3" s="21" t="str">
         <x:v>Calendar companion | October 19 to November 28, 2026</x:v>
       </x:c>
-      <x:c r="B3" s="18"/>
-      <x:c r="C3" s="18"/>
-      <x:c r="D3" s="18"/>
-      <x:c r="E3" s="18"/>
-      <x:c r="F3" s="18"/>
-      <x:c r="G3" s="18"/>
+      <x:c r="B3" s="21"/>
+      <x:c r="C3" s="21"/>
+      <x:c r="D3" s="21"/>
+      <x:c r="E3" s="21"/>
+      <x:c r="F3" s="21"/>
+      <x:c r="G3" s="21"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="28" t="str">
+      <x:c r="A5" s="29" t="str">
         <x:v>Target date</x:v>
       </x:c>
-      <x:c r="B5" s="28" t="str">
+      <x:c r="B5" s="29" t="str">
         <x:v>Assignment</x:v>
       </x:c>
-      <x:c r="C5" s="28" t="str">
+      <x:c r="C5" s="29" t="str">
         <x:v>Audience and send gate</x:v>
       </x:c>
-      <x:c r="D5" s="28" t="str">
+      <x:c r="D5" s="29" t="str">
         <x:v>Hub destination</x:v>
       </x:c>
-      <x:c r="E5" s="28" t="str">
+      <x:c r="E5" s="29" t="str">
         <x:v>Creative and next action</x:v>
       </x:c>
-      <x:c r="F5" s="28" t="str">
+      <x:c r="F5" s="29" t="str">
         <x:v>Measurement</x:v>
       </x:c>
-      <x:c r="G5" s="28" t="str">
+      <x:c r="G5" s="29" t="str">
         <x:v>Status</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="112" customHeight="1">
-      <x:c r="A6" s="29" t="str">
+      <x:c r="A6" s="30" t="str">
         <x:v>Oct 30</x:v>
       </x:c>
-      <x:c r="B6" s="29" t="str">
+      <x:c r="B6" s="30" t="str">
         <x:v>Rug care return email</x:v>
       </x:c>
-      <x:c r="C6" s="29" t="str">
+      <x:c r="C6" s="30" t="str">
         <x:v>Relevant existing customers or subscribers, if a suitable segment exists. Check Constant Contact schedule and suppress duplicates before sending.</x:v>
       </x:c>
-      <x:c r="D6" s="29" t="str">
+      <x:c r="D6" s="30" t="str">
         <x:v>October 29 Oriental rug evaluation guide, exact live permalink</x:v>
       </x:c>
-      <x:c r="E6" s="29" t="str">
+      <x:c r="E6" s="30" t="str">
         <x:v>Use a recognizable person + Aladdin sender, a specific subject and conversational plain text with no logo/header. Answer one rug-care question; link to the guide and its verified contact action.</x:v>
       </x:c>
-      <x:c r="F6" s="29" t="str">
+      <x:c r="F6" s="30" t="str">
         <x:v>Delivered, unsubscribes, clicks, tagged article sessions, separate form/phone events and qualified inquiries. Do not equate clicks with visits.</x:v>
       </x:c>
-      <x:c r="G6" s="29" t="str">
+      <x:c r="G6" s="30" t="str">
         <x:v>Planned test; send date and audience require schedule review</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="112" customHeight="1">
-      <x:c r="A7" s="29" t="str">
+      <x:c r="A7" s="30" t="str">
         <x:v>Nov 20</x:v>
       </x:c>
-      <x:c r="B7" s="29" t="str">
+      <x:c r="B7" s="30" t="str">
         <x:v>Pre-guest care return email</x:v>
       </x:c>
-      <x:c r="C7" s="29" t="str">
+      <x:c r="C7" s="30" t="str">
         <x:v>Conditional: review first email relevance, clicks, tagged visits, inquiries and unsubscribes; check existing sends and availability before proceeding.</x:v>
       </x:c>
-      <x:c r="D7" s="29" t="str">
+      <x:c r="D7" s="30" t="str">
         <x:v>November 19 practical pre-guest care guide, exact live permalink</x:v>
       </x:c>
-      <x:c r="E7" s="29" t="str">
+      <x:c r="E7" s="30" t="str">
         <x:v>Use the same person + company, specific subject and plain-text approach. Offer a useful planning answer without holiday urgency or unverified availability.</x:v>
       </x:c>
-      <x:c r="F7" s="29" t="str">
+      <x:c r="F7" s="30" t="str">
         <x:v>Delivered, unsubscribes, clicks, tagged guide sessions, separate form/phone events and qualified inquiries.</x:v>
       </x:c>
-      <x:c r="G7" s="29" t="str">
+      <x:c r="G7" s="30" t="str">
         <x:v>Conditional planned test</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="26"/>
-      <x:c r="B8" s="26"/>
-      <x:c r="C8" s="26"/>
-      <x:c r="D8" s="26"/>
-      <x:c r="E8" s="26"/>
-      <x:c r="F8" s="26"/>
-      <x:c r="G8" s="26"/>
+      <x:c r="A8" s="17"/>
+      <x:c r="B8" s="17"/>
+      <x:c r="C8" s="17"/>
+      <x:c r="D8" s="17"/>
+      <x:c r="E8" s="17"/>
+      <x:c r="F8" s="17"/>
+      <x:c r="G8" s="17"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="27" t="str">
+      <x:c r="A9" s="28" t="str">
         <x:v>Weekly measurement and publishing checks</x:v>
       </x:c>
-      <x:c r="B9" s="27"/>
-      <x:c r="C9" s="27"/>
-      <x:c r="D9" s="27"/>
-      <x:c r="E9" s="27"/>
-      <x:c r="F9" s="27"/>
-      <x:c r="G9" s="27"/>
+      <x:c r="B9" s="28"/>
+      <x:c r="C9" s="28"/>
+      <x:c r="D9" s="28"/>
+      <x:c r="E9" s="28"/>
+      <x:c r="F9" s="28"/>
+      <x:c r="G9" s="28"/>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
-      <x:c r="A10" s="28" t="str">
+      <x:c r="A10" s="29" t="str">
         <x:v>Check</x:v>
       </x:c>
-      <x:c r="B10" s="28" t="str">
+      <x:c r="B10" s="29" t="str">
         <x:v>Record separately</x:v>
       </x:c>
-      <x:c r="C10" s="28" t="str">
+      <x:c r="C10" s="29" t="str">
         <x:v>Decision rule</x:v>
       </x:c>
-      <x:c r="D10" s="26"/>
-      <x:c r="E10" s="26"/>
-      <x:c r="F10" s="26"/>
-      <x:c r="G10" s="26"/>
+      <x:c r="D10" s="17"/>
+      <x:c r="E10" s="17"/>
+      <x:c r="F10" s="17"/>
+      <x:c r="G10" s="17"/>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
-      <x:c r="A11" s="29" t="str">
+      <x:c r="A11" s="30" t="str">
         <x:v>Link path</x:v>
       </x:c>
-      <x:c r="B11" s="29" t="str">
+      <x:c r="B11" s="30" t="str">
         <x:v>Post/email ID, tagged URL, article or service landing page, CTA and final contact path</x:v>
       </x:c>
-      <x:c r="C11" s="29" t="str">
+      <x:c r="C11" s="30" t="str">
         <x:v>Facebook links to the exact matching Aladdin page; email links to the hub; Instagram caption uses 210-361-3930, without a raw URL.</x:v>
       </x:c>
-      <x:c r="D11" s="26"/>
-      <x:c r="E11" s="26"/>
-      <x:c r="F11" s="26"/>
-      <x:c r="G11" s="26"/>
+      <x:c r="D11" s="17"/>
+      <x:c r="E11" s="17"/>
+      <x:c r="F11" s="17"/>
+      <x:c r="G11" s="17"/>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="A12" s="30" t="str">
         <x:v>Website response</x:v>
       </x:c>
-      <x:c r="B12" s="29" t="str">
+      <x:c r="B12" s="30" t="str">
         <x:v>Tagged sessions to each hub and contact path; form events; phone events</x:v>
       </x:c>
-      <x:c r="C12" s="29" t="str">
+      <x:c r="C12" s="30" t="str">
         <x:v>Verify event definitions after the Oct 19 tracking changes. Count forms and phone actions separately; inspect source and service fit.</x:v>
       </x:c>
-      <x:c r="D12" s="26"/>
-      <x:c r="E12" s="26"/>
-      <x:c r="F12" s="26"/>
-      <x:c r="G12" s="26"/>
+      <x:c r="D12" s="17"/>
+      <x:c r="E12" s="17"/>
+      <x:c r="F12" s="17"/>
+      <x:c r="G12" s="17"/>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
-      <x:c r="A13" s="29" t="str">
+      <x:c r="A13" s="30" t="str">
         <x:v>Lead quality</x:v>
       </x:c>
-      <x:c r="B13" s="29" t="str">
+      <x:c r="B13" s="30" t="str">
         <x:v>Real submissions, qualified inquiries, estimates and booked work when available</x:v>
       </x:c>
-      <x:c r="C13" s="29" t="str">
+      <x:c r="C13" s="30" t="str">
         <x:v>Exclude marked tests; do not treat GA4 events or phone taps as unique customers or completed calls.</x:v>
       </x:c>
-      <x:c r="D13" s="26"/>
-      <x:c r="E13" s="26"/>
-      <x:c r="F13" s="26"/>
-      <x:c r="G13" s="26"/>
+      <x:c r="D13" s="17"/>
+      <x:c r="E13" s="17"/>
+      <x:c r="F13" s="17"/>
+      <x:c r="G13" s="17"/>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
-      <x:c r="A14" s="29" t="str">
+      <x:c r="A14" s="30" t="str">
         <x:v>Email response</x:v>
       </x:c>
-      <x:c r="B14" s="29" t="str">
+      <x:c r="B14" s="30" t="str">
         <x:v>Delivered, clicks, tagged return sessions, inquiries and unsubscribes</x:v>
       </x:c>
-      <x:c r="C14" s="29" t="str">
+      <x:c r="C14" s="30" t="str">
         <x:v>Clicks rose in the report, but unsubscribes rose too. Review the first send before a second or any increase in frequency.</x:v>
       </x:c>
-      <x:c r="D14" s="26"/>
-      <x:c r="E14" s="26"/>
-      <x:c r="F14" s="26"/>
-      <x:c r="G14" s="26"/>
+      <x:c r="D14" s="17"/>
+      <x:c r="E14" s="17"/>
+      <x:c r="F14" s="17"/>
+      <x:c r="G14" s="17"/>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
-      <x:c r="A15" s="29" t="str">
+      <x:c r="A15" s="30" t="str">
         <x:v>Comparison</x:v>
       </x:c>
-      <x:c r="B15" s="29" t="str">
+      <x:c r="B15" s="30" t="str">
         <x:v>Matched publication age, format, exposure, source and post-change reporting period</x:v>
       </x:c>
-      <x:c r="C15" s="29" t="str">
+      <x:c r="C15" s="30" t="str">
         <x:v>The two PDFs use different dates, and measurement changed Oct 19. Do not claim uplift from one blended baseline.</x:v>
       </x:c>
-      <x:c r="D15" s="26"/>
-      <x:c r="E15" s="26"/>
-      <x:c r="F15" s="26"/>
-      <x:c r="G15" s="26"/>
+      <x:c r="D15" s="17"/>
+      <x:c r="E15" s="17"/>
+      <x:c r="F15" s="17"/>
+      <x:c r="G15" s="17"/>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
-      <x:c r="A16" s="29" t="str">
+      <x:c r="A16" s="30" t="str">
         <x:v>Service fit</x:v>
       </x:c>
-      <x:c r="B16" s="29" t="str">
+      <x:c r="B16" s="30" t="str">
         <x:v>Relevant service area and actual customer problem when available</x:v>
       </x:c>
-      <x:c r="C16" s="29" t="str">
+      <x:c r="C16" s="30" t="str">
         <x:v>Geography is approximate and filtering is off; do not assume every session is a local prospect or a bot.</x:v>
       </x:c>
-      <x:c r="D16" s="26"/>
-      <x:c r="E16" s="26"/>
-      <x:c r="F16" s="26"/>
-      <x:c r="G16" s="26"/>
+      <x:c r="D16" s="17"/>
+      <x:c r="E16" s="17"/>
+      <x:c r="F16" s="17"/>
+      <x:c r="G16" s="17"/>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
-      <x:c r="A17" s="29" t="str">
+      <x:c r="A17" s="30" t="str">
         <x:v>Publishing gate</x:v>
       </x:c>
-      <x:c r="B17" s="29" t="str">
+      <x:c r="B17" s="30" t="str">
         <x:v>Live permalink, service-specific CTA, responsive contact action, image and claims approval</x:v>
       </x:c>
-      <x:c r="C17" s="29" t="str">
+      <x:c r="C17" s="30" t="str">
         <x:v>Use the current Strategy Canvas and voice; obtain operations approval for emergency/insurance claims and named assessment offers.</x:v>
       </x:c>
-      <x:c r="D17" s="26"/>
-      <x:c r="E17" s="26"/>
-      <x:c r="F17" s="26"/>
-      <x:c r="G17" s="26"/>
+      <x:c r="D17" s="17"/>
+      <x:c r="E17" s="17"/>
+      <x:c r="F17" s="17"/>
+      <x:c r="G17" s="17"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Connect Aladdin social, blog, email and inquiry paths in 45-day calendar
</commit_message>
<xml_diff>
--- a/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
+++ b/clients/aladdin/calendar/Aladdin-Next-45-Day-Organic-Calendar-2026-10-15-to-11-28.xlsx
@@ -2,12 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="Rb5873ca60583419b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="R52bce0fce8d44093"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="R8f41fb63186041b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="Re24811e01c9143fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="R78e1a5a8047e43bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email and Measurement" sheetId="6" r:id="R0d4dab93e5894815"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Summary" sheetId="1" r:id="R4be372ff497749d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45-Day Calendar" sheetId="2" r:id="Re4854849809a48ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Message Matrix" sheetId="3" r:id="Rb61f3e17250d4fdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Campaign Matrix" sheetId="4" r:id="R50ed04d377514fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Guardrails" sheetId="5" r:id="Rfdee5228007445db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email and Measurement" sheetId="6" r:id="R0292f9b561e64158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Post Path Map" sheetId="7" r:id="Rd60d42de2f2142b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connected Content Briefs" sheetId="8" r:id="Rc37ab06bd35d4453"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Email Drafts" sheetId="9" r:id="Rc81fda439ee44c62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +24,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="mm/dd/yy"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -90,8 +93,19 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -111,6 +125,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7F2EC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF9D1725"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9E4DD"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF9D1725"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9E4DD"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -160,7 +194,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -226,6 +260,36 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -752,6 +816,22 @@
         <x:v>Keep the four Strategy Canvas paths, Aladdin voice, photo-led assets and channel-specific CTAs. Verify live permalinks, service scope, uniform colors and emergency claims before scheduling.</x:v>
       </x:c>
     </x:row>
+    <x:row r="39" ht="62" customHeight="1">
+      <x:c r="A39" s="38" t="str">
+        <x:v>Reader paths</x:v>
+      </x:c>
+      <x:c r="B39" s="16" t="str">
+        <x:v>Use the Post Path Map to check the route from each post or email to its exact website destination and on to the proper form, call action or gallery purchase page. Saved scheduled posts require a separate CoSchedule check; future article links remain gated until publication.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="72" customHeight="1">
+      <x:c r="A40" s="38" t="str">
+        <x:v>Content integration</x:v>
+      </x:c>
+      <x:c r="B40" s="16" t="str">
+        <x:v>Future planned posts now form rug, upholstery, water-response and pre-guest sequences. Each sequence has a useful social promise, a specific website guide, the correct form or call handoff, and an email or deliberate no-email choice. See Connected Content Briefs and Email Drafts.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1523,10 +1603,10 @@
         <x:v>Specialty Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str">
-        <x:v>When is a rug worth a closer evaluation?</x:v>
+        <x:v>Five clues your rug deserves a closer look before cleaning</x:v>
       </x:c>
       <x:c r="I17" s="6" t="str">
-        <x:v>Saveable cues: sentimental value, unknown material, color movement, previous repair or persistent concern. Avoid fear or promised outcomes.</x:v>
+        <x:v>Photo carousel: show real rug details, not a text card. Slides: label or provenance, fiber/construction, color movement, prior repair, and a final question about uncertainty. Give one useful observation per slide; do not diagnose from a photo. Facebook points to the rug-care page; the Oct 29 article deepens the decision.</x:v>
       </x:c>
       <x:c r="J17" s="6" t="str">
         <x:v>Photo carousel</x:v>
@@ -1535,10 +1615,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L17" s="6" t="str">
-        <x:v>Save / ask about your rug</x:v>
+        <x:v>See how Aladdin approaches rug care / ask about your rug</x:v>
       </x:c>
       <x:c r="M17" s="6" t="str">
-        <x:v>Oriental rugs page</x:v>
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
       </x:c>
       <x:c r="N17" s="6" t="str">
         <x:v>Real rug details; condition claims verified</x:v>
@@ -1579,10 +1659,10 @@
         <x:v>Expertise / Inside the Craft</x:v>
       </x:c>
       <x:c r="H18" s="6" t="str">
-        <x:v>What an intake can reveal</x:v>
+        <x:v>What happens when Aladdin first examines a rug?</x:v>
       </x:c>
       <x:c r="I18" s="6" t="str">
-        <x:v>Show documented rug intake and the questions that guide the care plan. Do not present a staged scene as an actual customer job.</x:v>
+        <x:v>Short footage or approved photos of intake: listen to the owner, document condition, examine construction and dye concerns, then explain options. End with the question a customer can bring to a first conversation. Link Facebook to rug care; use this as a bridge to the Oct 29 guide.</x:v>
       </x:c>
       <x:c r="J18" s="6" t="str">
         <x:v>Short process video</x:v>
@@ -1591,10 +1671,10 @@
         <x:v>Instagram Reel + Facebook</x:v>
       </x:c>
       <x:c r="L18" s="6" t="str">
-        <x:v>Ask how your rug would be evaluated</x:v>
+        <x:v>See the rug-care process / ask a question</x:v>
       </x:c>
       <x:c r="M18" s="6" t="str">
-        <x:v>Rug cleaning page</x:v>
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
       </x:c>
       <x:c r="N18" s="6" t="str">
         <x:v>Approved facility footage; verify actual sequence and credentials</x:v>
@@ -1635,10 +1715,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H19" s="6" t="str">
-        <x:v>What do you know about your rug?</x:v>
+        <x:v>What would you want to know before a rug is cleaned?</x:v>
       </x:c>
       <x:c r="I19" s="6" t="str">
-        <x:v>Invite questions about material, construction, age or past care; advise assessment when uncertain.</x:v>
+        <x:v>Ask for one specific uncertainty: age, fiber, dye, old repair or previous cleaning. Answer one common response with a factual teaser to tomorrow’s evaluation guide. Do not request personal details in comments.</x:v>
       </x:c>
       <x:c r="J19" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -1647,10 +1727,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L19" s="6" t="str">
-        <x:v>Send a general rug question</x:v>
+        <x:v>Ask a rug question / return for tomorrow’s guide</x:v>
       </x:c>
       <x:c r="M19" s="6" t="str">
-        <x:v>Rug cleaning page on October 28; October 29 guide only after publication</x:v>
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
       </x:c>
       <x:c r="N19" s="6" t="str">
         <x:v>Actual rug close-up; no unsupported diagnosis Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
@@ -1691,10 +1771,10 @@
         <x:v>Specialty Care / Inside the Craft</x:v>
       </x:c>
       <x:c r="H20" s="6" t="str">
-        <x:v>What an Oriental rug evaluation should cover</x:v>
+        <x:v>Before cleaning an Oriental rug, what should be evaluated?</x:v>
       </x:c>
       <x:c r="I20" s="6" t="str">
-        <x:v>Hub guide on rug history, fiber/construction, condition, dyes, prior repairs and realistic next steps.</x:v>
+        <x:v>Publish a useful owner-facing article covering rug history, construction, fiber and dye, existing condition, old repairs, and what can and cannot be known before work. Include a clear rug-care inquiry route to the improved residential form and a phone option. Social excerpt answers one question and invites the reader to the full guide.</x:v>
       </x:c>
       <x:c r="J20" s="6" t="str">
         <x:v>Blog + social excerpts</x:v>
@@ -1703,7 +1783,7 @@
         <x:v>Website + Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L20" s="6" t="str">
-        <x:v>Read the guide / discuss your rug with Aladdin</x:v>
+        <x:v>Read the evaluation guide / ask Aladdin about your rug</x:v>
       </x:c>
       <x:c r="M20" s="6" t="str">
         <x:v>October 29 rug evaluation guide; publish first, then use exact permalink</x:v>
@@ -1747,10 +1827,10 @@
         <x:v>Trust &amp; Legacy / San Antonio Stories</x:v>
       </x:c>
       <x:c r="H21" s="6" t="str">
-        <x:v>Choosing a rug is personal</x:v>
+        <x:v>A one-of-a-kind rug should fit the room and the buyer</x:v>
       </x:c>
       <x:c r="I21" s="6" t="str">
-        <x:v>Use the Rug Gallery to show how size, condition and room context matter. Highlight a real piece only after rechecking inventory and price.</x:v>
+        <x:v>Use several real, currently available Rug Gallery photos showing distinct styles and prices. Explain size, condition, color and room use as purchase considerations. Link a verified product or gallery page; keep shopping metrics distinct from service leads.</x:v>
       </x:c>
       <x:c r="J21" s="6" t="str">
         <x:v>Product photo story</x:v>
@@ -1759,10 +1839,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L21" s="6" t="str">
-        <x:v>Explore the gallery / call with a question</x:v>
+        <x:v>Explore available rugs in the Gallery</x:v>
       </x:c>
       <x:c r="M21" s="6" t="str">
-        <x:v>Current Rug Gallery or verified product page</x:v>
+        <x:v>https://aladdincleans.com/rug-store/</x:v>
       </x:c>
       <x:c r="N21" s="6" t="str">
         <x:v>Authentic product photo; recheck inventory, price, rights</x:v>
@@ -1803,10 +1883,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H22" s="6" t="str">
-        <x:v>After the rug evaluation guide, what would you ask next?</x:v>
+        <x:v>What should you ask after reading the rug evaluation guide?</x:v>
       </x:c>
       <x:c r="I22" s="6" t="str">
-        <x:v>Follow the October 29 guide with a specific question about material, dye, condition or prior repair. Answer one concern from the article, then invite readers to the full guide. Facebook links to the exact live permalink; Instagram keeps the phone CTA.</x:v>
+        <x:v>Recap three owner questions from the Oct 29 article: what is known, what needs inspection and which outcome matters most. Link the exact article in Facebook only after publication; Instagram gives a concise question plus approved phone CTA. Invite an inquiry through the article’s form route.</x:v>
       </x:c>
       <x:c r="J22" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -1815,7 +1895,7 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L22" s="6" t="str">
-        <x:v>Read the rug evaluation guide / ask about your rug</x:v>
+        <x:v>Read the guide / ask a rug-care question</x:v>
       </x:c>
       <x:c r="M22" s="6" t="str">
         <x:v>October 29 rug evaluation guide, exact permalink after publication</x:v>
@@ -1915,10 +1995,10 @@
         <x:v>Complete Property Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H24" s="6" t="str">
-        <x:v>Three questions before upholstery care</x:v>
+        <x:v>Before upholstery cleaning, ask these three questions</x:v>
       </x:c>
       <x:c r="I24" s="6" t="str">
-        <x:v>Ask about material, use and existing concerns before choosing a method. Invite assessment rather than blanket advice.</x:v>
+        <x:v>Photo-led carousel: what is the fabric, what changed, and what result matters? Explain why the answers guide a conversation rather than promising a uniform method. Link the upholstery page; promise a fuller owner guide on Nov 5.</x:v>
       </x:c>
       <x:c r="J24" s="6" t="str">
         <x:v>Photo carousel</x:v>
@@ -1927,10 +2007,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L24" s="6" t="str">
-        <x:v>Save / ask about upholstery</x:v>
+        <x:v>Explore upholstery care / ask about your furniture</x:v>
       </x:c>
       <x:c r="M24" s="6" t="str">
-        <x:v>Upholstery cleaning page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
       </x:c>
       <x:c r="N24" s="6" t="str">
         <x:v>Real textile photos; avoid stain-removal guarantees</x:v>
@@ -1971,10 +2051,10 @@
         <x:v>Expertise / Inside the Craft</x:v>
       </x:c>
       <x:c r="H25" s="6" t="str">
-        <x:v>How a fabric question becomes a care plan</x:v>
+        <x:v>Why the fabric label is only the start of the conversation</x:v>
       </x:c>
       <x:c r="I25" s="6" t="str">
-        <x:v>Short process story: listen, inspect, explain options, set expectations.</x:v>
+        <x:v>Use approved process photos to show listening, inspection, explanation and realistic expectations. Give one example question to bring to a visit. Link upholstery care and lead into the Nov 5 guide.</x:v>
       </x:c>
       <x:c r="J25" s="6" t="str">
         <x:v>Short process video</x:v>
@@ -1983,10 +2063,10 @@
         <x:v>Instagram Reel + Facebook</x:v>
       </x:c>
       <x:c r="L25" s="6" t="str">
-        <x:v>Ask what care fits your furniture</x:v>
+        <x:v>See Aladdin’s upholstery approach</x:v>
       </x:c>
       <x:c r="M25" s="6" t="str">
-        <x:v>Upholstery cleaning page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
       </x:c>
       <x:c r="N25" s="6" t="str">
         <x:v>Approved technician footage; uniform and process check</x:v>
@@ -2027,10 +2107,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H26" s="6" t="str">
-        <x:v>Which surface do you have a question about?</x:v>
+        <x:v>Which furniture-care question should the guide answer?</x:v>
       </x:c>
       <x:c r="I26" s="6" t="str">
-        <x:v>Let households choose upholstery, rugs, carpet or hard floors. Use replies to guide practical content.</x:v>
+        <x:v>Poll for material, stains, wear or drying concerns. Use the winning question as a short introduction in tomorrow’s guide if editorial timing allows. Facebook links to the current upholstery page until the new article is live.</x:v>
       </x:c>
       <x:c r="J26" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2039,10 +2119,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L26" s="6" t="str">
-        <x:v>Vote</x:v>
+        <x:v>Vote / read the upholstery guide tomorrow</x:v>
       </x:c>
       <x:c r="M26" s="6" t="str">
-        <x:v>Upholstery page on November 4; November 5 guide only after publication</x:v>
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
       </x:c>
       <x:c r="N26" s="6" t="str">
         <x:v>Four real surface photos; no icon-only card Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
@@ -2083,10 +2163,10 @@
         <x:v>Complete Property Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H27" s="6" t="str">
-        <x:v>A practical upholstery care conversation</x:v>
+        <x:v>How to plan upholstery care without guessing</x:v>
       </x:c>
       <x:c r="I27" s="6" t="str">
-        <x:v>Hub guide on material, condition, expectations and timing; connect to the wider home only when useful.</x:v>
+        <x:v>Publish the Nov 5 guide: fabric and construction, current condition, household use, realistic outcomes, timing and aftercare questions. Add the appropriate residential inquiry form and phone CTA. Social posts give one useful answer and a reason to read the full guide.</x:v>
       </x:c>
       <x:c r="J27" s="6" t="str">
         <x:v>Blog + social excerpts</x:v>
@@ -2095,7 +2175,7 @@
         <x:v>Website + Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L27" s="6" t="str">
-        <x:v>Read the guide / request residential care</x:v>
+        <x:v>Read the upholstery guide / request a conversation</x:v>
       </x:c>
       <x:c r="M27" s="6" t="str">
         <x:v>November 5 upholstery guide; publish first, then use exact permalink</x:v>
@@ -2139,10 +2219,10 @@
         <x:v>Customer Experience / Proof With Context</x:v>
       </x:c>
       <x:c r="H28" s="6" t="str">
-        <x:v>Why careful recommendations matter</x:v>
+        <x:v>What careful upholstery advice sounds like</x:v>
       </x:c>
       <x:c r="I28" s="6" t="str">
-        <x:v>Use a real approved example of explaining options and respecting a customer’s priorities; no invented result.</x:v>
+        <x:v>Use only an approved, specific customer or team example: the concern, question asked, option explained and realistic expectation. Link back to the Nov 5 guide once live; no invented testimonial or result claim.</x:v>
       </x:c>
       <x:c r="J28" s="6" t="str">
         <x:v>Photo story</x:v>
@@ -2151,10 +2231,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L28" s="6" t="str">
-        <x:v>See Aladdin’s approach / call</x:v>
+        <x:v>Read the guide / ask about your furniture</x:v>
       </x:c>
       <x:c r="M28" s="6" t="str">
-        <x:v>About or upholstery page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
       </x:c>
       <x:c r="N28" s="6" t="str">
         <x:v>Customer permission if identifiable; actual team photo</x:v>
@@ -2198,7 +2278,7 @@
         <x:v>What would you ask about a favorite chair?</x:v>
       </x:c>
       <x:c r="I29" s="6" t="str">
-        <x:v>Light Story question that surfaces material and care concerns.</x:v>
+        <x:v>Story question follows the Nov 5 guide: material, condition, timing or result. Share a useful anonymized answer later. The article carries the inquiry path; do not force a link into a platform-only Story.</x:v>
       </x:c>
       <x:c r="J29" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2207,7 +2287,7 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L29" s="6" t="str">
-        <x:v>Reply</x:v>
+        <x:v>Reply with a chair-care question</x:v>
       </x:c>
       <x:c r="M29" s="6" t="str">
         <x:v>Upholstery page</x:v>
@@ -2307,10 +2387,10 @@
         <x:v>Expertise / Protect What Matters</x:v>
       </x:c>
       <x:c r="H31" s="6" t="str">
-        <x:v>What to know before water affects a room</x:v>
+        <x:v>Water in a room: what is useful to know first?</x:v>
       </x:c>
       <x:c r="I31" s="6" t="str">
-        <x:v>Saveable checklist: safety first, document what is visible from a safe place, and know where to find the appropriate contact. Never tell readers to enter an unsafe area.</x:v>
+        <x:v>Operations-approved, photo-led checklist: personal safety, document what can be seen safely, know who to call and share relevant access details. Avoid prescriptive cleanup or response-time claims. Facebook links to current restoration guidance; Instagram offers the confirmed active-issue call route.</x:v>
       </x:c>
       <x:c r="J31" s="6" t="str">
         <x:v>Photo carousel</x:v>
@@ -2319,10 +2399,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L31" s="6" t="str">
-        <x:v>Save the steps / seek qualified guidance</x:v>
+        <x:v>Read restoration guidance / call for an active issue</x:v>
       </x:c>
       <x:c r="M31" s="6" t="str">
-        <x:v>Water-damage restoration page</x:v>
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
       </x:c>
       <x:c r="N31" s="6" t="str">
         <x:v>Verify safety language and confirmed contact path with restoration operations</x:v>
@@ -2363,10 +2443,10 @@
         <x:v>Expertise / Inside the Craft</x:v>
       </x:c>
       <x:c r="H32" s="6" t="str">
-        <x:v>What a useful incident record includes</x:v>
+        <x:v>Four details that help the first water-damage conversation</x:v>
       </x:c>
       <x:c r="I32" s="6" t="str">
-        <x:v>Show how clear photos, timing, contacts and site access information can help the first conversation; do not promise an insurance result.</x:v>
+        <x:v>Use a facility or home scenario: when noticed, affected area, safe photos and access/contact person. Explain that this record helps the initial conversation without promising an outcome. Point to current restoration guidance and the Nov 12 article.</x:v>
       </x:c>
       <x:c r="J32" s="6" t="str">
         <x:v>Document/photo feed</x:v>
@@ -2375,10 +2455,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L32" s="6" t="str">
-        <x:v>Share with your facilities team</x:v>
+        <x:v>Save the checklist / see current restoration guidance</x:v>
       </x:c>
       <x:c r="M32" s="6" t="str">
-        <x:v>Water-damage restoration page</x:v>
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
       </x:c>
       <x:c r="N32" s="6" t="str">
         <x:v>No customer records or private site details; operations review required</x:v>
@@ -2419,10 +2499,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H33" s="6" t="str">
-        <x:v>What should you document after water enters a room?</x:v>
+        <x:v>After water enters a room, what should you document?</x:v>
       </x:c>
       <x:c r="I33" s="6" t="str">
-        <x:v>Use one practical, operations-approved documentation question as the lead-in to the November 12 guide. Refer an active water or fire issue to the confirmed emergency phone path; do not imply a public comment is triage.</x:v>
+        <x:v>Ask one practical question, then answer it with an operations-approved list. This is the bridge to tomorrow’s guide. Facebook links to the current water page until the article is live; active issues use the verified call route.</x:v>
       </x:c>
       <x:c r="J33" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2431,10 +2511,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L33" s="6" t="str">
-        <x:v>Read current restoration guidance / call for active help</x:v>
+        <x:v>Read current guidance / call for active help</x:v>
       </x:c>
       <x:c r="M33" s="6" t="str">
-        <x:v>Water-damage restoration page on November 11; November 12 guide only after publication</x:v>
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
       </x:c>
       <x:c r="N33" s="6" t="str">
         <x:v>Operations and compliance approval of safety and response language; verify emergency number and live permalink</x:v>
@@ -2475,10 +2555,10 @@
         <x:v>Expertise / Protect What Matters</x:v>
       </x:c>
       <x:c r="H34" s="6" t="str">
-        <x:v>What a clear water-damage response should explain</x:v>
+        <x:v>A calmer first conversation after water damage</x:v>
       </x:c>
       <x:c r="I34" s="6" t="str">
-        <x:v>Hub guide on safe first steps, what to document, what triage can determine and which decisions require an on-site assessment. No claim about coverage, drying time or guaranteed response.</x:v>
+        <x:v>Publish an operations-reviewed guide: safety, documentation, who needs to be contacted, what an initial assessment may clarify and what remains uncertain. Give an unmistakable call action for active situations; do not send urgent readers through the residential cleaning form. Social excerpt summarizes one helpful step and links to the article.</x:v>
       </x:c>
       <x:c r="J34" s="6" t="str">
         <x:v>Blog + social excerpts</x:v>
@@ -2531,10 +2611,10 @@
         <x:v>Customer Experience / Proof With Context</x:v>
       </x:c>
       <x:c r="H35" s="6" t="str">
-        <x:v>The people behind a calm response</x:v>
+        <x:v>What a calm response sounds like from the team</x:v>
       </x:c>
       <x:c r="I35" s="6" t="str">
-        <x:v>Use an approved team photo and one verified communication practice from restoration operations.</x:v>
+        <x:v>Use an approved actual team photo and a verified practice such as clarifying contacts and next steps. Link to the Nov 12 guide after publication. No unsupported emergency availability claim.</x:v>
       </x:c>
       <x:c r="J35" s="6" t="str">
         <x:v>Team photo feed</x:v>
@@ -2543,10 +2623,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L35" s="6" t="str">
-        <x:v>Meet the team / call with a question</x:v>
+        <x:v>Read the response guide / call with a question</x:v>
       </x:c>
       <x:c r="M35" s="6" t="str">
-        <x:v>About or restoration page</x:v>
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
       </x:c>
       <x:c r="N35" s="6" t="str">
         <x:v>Employee permission; verified role; correct uniform; no invented response claim</x:v>
@@ -2587,10 +2667,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H36" s="6" t="str">
-        <x:v>Who has the first call and site access?</x:v>
+        <x:v>Before a facility closes, who can give access?</x:v>
       </x:c>
       <x:c r="I36" s="6" t="str">
-        <x:v>Ask facility teams to check current contacts and access roles before an incident; refer active emergencies to the confirmed contact path.</x:v>
+        <x:v>Ask commercial decision makers to confirm who receives the first call, who can open the property and where current site details live. Link the commercial page; the Nov 12 guide supplies documentation context.</x:v>
       </x:c>
       <x:c r="J36" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2599,10 +2679,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L36" s="6" t="str">
-        <x:v>Check your plan / ask Aladdin</x:v>
+        <x:v>Review your facility contact plan</x:v>
       </x:c>
       <x:c r="M36" s="6" t="str">
-        <x:v>Commercial services page</x:v>
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
       </x:c>
       <x:c r="N36" s="6" t="str">
         <x:v>No guarantee of availability or response time</x:v>
@@ -2699,10 +2779,10 @@
         <x:v>Complete Property Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H38" s="6" t="str">
-        <x:v>Plan the spaces that matter before guests arrive</x:v>
+        <x:v>Before guests arrive, choose the spaces that matter</x:v>
       </x:c>
       <x:c r="I38" s="6" t="str">
-        <x:v>Saveable checklist based on actual use, material condition and realistic timing. Avoid pressure or a whole-house upsell.</x:v>
+        <x:v>Photo-led checklist: identify high-use spaces, fragile materials and a realistic date to discuss service. Give one example of priorities to share with Aladdin. Link residential services and point to the Nov 19 planning guide.</x:v>
       </x:c>
       <x:c r="J38" s="6" t="str">
         <x:v>Photo carousel</x:v>
@@ -2711,10 +2791,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L38" s="6" t="str">
-        <x:v>Save the plan / ask about priorities</x:v>
+        <x:v>See residential care / ask about timing</x:v>
       </x:c>
       <x:c r="M38" s="6" t="str">
-        <x:v>Residential services page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
       </x:c>
       <x:c r="N38" s="6" t="str">
         <x:v>Warm real home photos; no staged client claim</x:v>
@@ -2755,10 +2835,10 @@
         <x:v>Customer Experience / Inside the Craft</x:v>
       </x:c>
       <x:c r="H39" s="6" t="str">
-        <x:v>How to prepare for a service visit</x:v>
+        <x:v>What should you tell Aladdin before a home visit?</x:v>
       </x:c>
       <x:c r="I39" s="6" t="str">
-        <x:v>Show practical access and communication steps customers can ask about before an appointment.</x:v>
+        <x:v>Show approved visit-prep photography: access, material concerns, priorities and questions. Explicitly mention that the improved form lets a visitor choose a service or “Not sure” and explain the need; do not imply service has been scheduled until confirmed.</x:v>
       </x:c>
       <x:c r="J39" s="6" t="str">
         <x:v>Short process video</x:v>
@@ -2767,10 +2847,10 @@
         <x:v>Instagram Reel + Facebook</x:v>
       </x:c>
       <x:c r="L39" s="6" t="str">
-        <x:v>Ask what to prepare</x:v>
+        <x:v>See how to request residential care</x:v>
       </x:c>
       <x:c r="M39" s="6" t="str">
-        <x:v>Schedule online or residential page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
       </x:c>
       <x:c r="N39" s="6" t="str">
         <x:v>Real service-prep footage; verify site guidance</x:v>
@@ -2811,10 +2891,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H40" s="6" t="str">
-        <x:v>Which room matters most when people gather?</x:v>
+        <x:v>Which room gets the most use when guests gather?</x:v>
       </x:c>
       <x:c r="I40" s="6" t="str">
-        <x:v>Poll on living area, dining area, entry or guest space. Invite priorities without suggesting all rooms need service.</x:v>
+        <x:v>Poll: living room, dining area, entry or guest space. Follow with one short planning consideration for the top answer; connect to the Nov 19 guide once published.</x:v>
       </x:c>
       <x:c r="J40" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2823,10 +2903,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L40" s="6" t="str">
-        <x:v>Vote</x:v>
+        <x:v>Vote / read the planning guide tomorrow</x:v>
       </x:c>
       <x:c r="M40" s="6" t="str">
-        <x:v>Residential services page on November 18; November 19 guide only after publication</x:v>
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
       </x:c>
       <x:c r="N40" s="6" t="str">
         <x:v>Real room photos; no icon-only card Feed format preserves caption CTAs; CoSchedule Stories do not send text.</x:v>
@@ -2867,10 +2947,10 @@
         <x:v>Complete Property Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H41" s="6" t="str">
-        <x:v>A calm pre-guest property-care plan</x:v>
+        <x:v>A practical home-care plan before guests arrive</x:v>
       </x:c>
       <x:c r="I41" s="6" t="str">
-        <x:v>Hub article: choose priorities, allow realistic lead time, protect specialty items and know when to leave a task for later.</x:v>
+        <x:v>Publish the Nov 19 guide: rank spaces, note material concerns, allow realistic lead time, prepare useful details for a service conversation and ask about timing. Link to the improved residential request form and phone. Social excerpt offers a mini checklist and invites the full plan.</x:v>
       </x:c>
       <x:c r="J41" s="6" t="str">
         <x:v>Blog + social excerpts</x:v>
@@ -2923,10 +3003,10 @@
         <x:v>Customer Experience / Proof With Context</x:v>
       </x:c>
       <x:c r="H42" s="6" t="str">
-        <x:v>Clear communication makes planning easier</x:v>
+        <x:v>Why clear expectations make a home visit easier</x:v>
       </x:c>
       <x:c r="I42" s="6" t="str">
-        <x:v>Use a real approved team or customer-experience detail about expectations before the visit.</x:v>
+        <x:v>Use an approved actual team image and one verified communication practice. Show which details a visitor can put in Special Requests and how the new “Not sure” service choice works. Link to the Nov 19 guide or residential form, as appropriate.</x:v>
       </x:c>
       <x:c r="J42" s="6" t="str">
         <x:v>Photo story</x:v>
@@ -2935,10 +3015,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L42" s="6" t="str">
-        <x:v>See what to expect / call</x:v>
+        <x:v>Read the plan / send your priorities</x:v>
       </x:c>
       <x:c r="M42" s="6" t="str">
-        <x:v>About or scheduling page</x:v>
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
       </x:c>
       <x:c r="N42" s="6" t="str">
         <x:v>Permission and claim check; no invented review</x:v>
@@ -2979,10 +3059,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H43" s="6" t="str">
-        <x:v>What is your last planning question?</x:v>
+        <x:v>What is still unclear about planning home care?</x:v>
       </x:c>
       <x:c r="I43" s="6" t="str">
-        <x:v>Light Story prompt about timing, access or material care.</x:v>
+        <x:v>Story prompt offers timing, materials and access as answer choices. Invite a question, then point interested readers to the Nov 19 guide through the platform link placement; Instagram caption keeps approved phone CTA.</x:v>
       </x:c>
       <x:c r="J43" s="6" t="str">
         <x:v>Photo question feed</x:v>
@@ -2991,7 +3071,7 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L43" s="6" t="str">
-        <x:v>Reply with a question</x:v>
+        <x:v>Reply with a planning question</x:v>
       </x:c>
       <x:c r="M43" s="6" t="str">
         <x:v>Pre-guest care guide</x:v>
@@ -3091,10 +3171,10 @@
         <x:v>Complete Property Care / Protect What Matters</x:v>
       </x:c>
       <x:c r="H45" s="6" t="str">
-        <x:v>Before a holiday closure, confirm the basics</x:v>
+        <x:v>Before a holiday closure, check these facility details</x:v>
       </x:c>
       <x:c r="I45" s="6" t="str">
-        <x:v>Checklist for contacts, access, responsibilities and known surface concerns. No emergency guarantee.</x:v>
+        <x:v>Commercial checklist: responsible contact, site access, known surface concerns and routine care priorities. Distinguish preparedness from an emergency promise. Facebook links to commercial services; Instagram uses a confirmed commercial contact action.</x:v>
       </x:c>
       <x:c r="J45" s="6" t="str">
         <x:v>Document/photo carousel</x:v>
@@ -3103,10 +3183,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L45" s="6" t="str">
-        <x:v>Save / share with your team</x:v>
+        <x:v>Review commercial service options</x:v>
       </x:c>
       <x:c r="M45" s="6" t="str">
-        <x:v>Commercial services page</x:v>
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
       </x:c>
       <x:c r="N45" s="6" t="str">
         <x:v>Actual commercial setting; no private site detail</x:v>
@@ -3147,10 +3227,10 @@
         <x:v>Expertise / Inside the Craft</x:v>
       </x:c>
       <x:c r="H46" s="6" t="str">
-        <x:v>A practical surface-care walkthrough</x:v>
+        <x:v>What does Aladdin need to know about a facility?</x:v>
       </x:c>
       <x:c r="I46" s="6" t="str">
-        <x:v>Explain how traffic areas, materials, access and recurring needs shape a facility conversation. Do not advertise an annual program until approved.</x:v>
+        <x:v>Approved photo/video walkthrough explains surface types, traffic, access windows and who approves a plan. Link commercial services; invite a useful first conversation rather than a generic quote request.</x:v>
       </x:c>
       <x:c r="J46" s="6" t="str">
         <x:v>Short process video</x:v>
@@ -3159,10 +3239,10 @@
         <x:v>Instagram Reel + Facebook</x:v>
       </x:c>
       <x:c r="L46" s="6" t="str">
-        <x:v>Ask about facility priorities</x:v>
+        <x:v>Ask about a facility-care plan</x:v>
       </x:c>
       <x:c r="M46" s="6" t="str">
-        <x:v>Commercial services page</x:v>
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
       </x:c>
       <x:c r="N46" s="6" t="str">
         <x:v>Real facility/process footage; verify service scope and capacity</x:v>
@@ -3315,10 +3395,10 @@
         <x:v>Expertise / Ask Aladdin</x:v>
       </x:c>
       <x:c r="H49" s="6" t="str">
-        <x:v>After a gathering, respond to a rug spill calmly</x:v>
+        <x:v>A rug spill after gathering: what should you do first?</x:v>
       </x:c>
       <x:c r="I49" s="6" t="str">
-        <x:v>Use existing verified spill guide: remove excess gently, blot, avoid experiments and seek material-specific guidance.</x:v>
+        <x:v>Reuse the verified Oct 15 rug-spill guide with a new, photo-led setup. Give one safe general point, then send Facebook readers to the exact article for limits and next steps. Verify the article’s form and phone route before scheduling.</x:v>
       </x:c>
       <x:c r="J49" s="6" t="str">
         <x:v>Photo feed</x:v>
@@ -3327,10 +3407,10 @@
         <x:v>Facebook + Instagram</x:v>
       </x:c>
       <x:c r="L49" s="6" t="str">
-        <x:v>Read the guide / call for guidance</x:v>
+        <x:v>Read the spill guide / call with a rug question</x:v>
       </x:c>
       <x:c r="M49" s="6" t="str">
-        <x:v>October 15 rug-spill article</x:v>
+        <x:v>https://aladdincleans.com/blog/oriental-rugs/what-to-do-first-after-a-spill-on-a-rug/</x:v>
       </x:c>
       <x:c r="N49" s="6" t="str">
         <x:v>Real rug/towel photo; recheck guide link and no outcome claims</x:v>
@@ -4228,6 +4308,26 @@
         <x:v>Aladdin-Cleaning-Restoration_Message-Magnet-Performance_2026-10-19_11-09-46_CT.pdf</x:v>
       </x:c>
     </x:row>
+    <x:row r="15" ht="90" customHeight="1">
+      <x:c r="A15" s="16" t="str">
+        <x:v>Live Aladdin path review, Oct 19</x:v>
+      </x:c>
+      <x:c r="B15" s="16" t="str">
+        <x:v>Current residential, rug, upholstery, water, commercial, gallery and request-page URLs</x:v>
+      </x:c>
+      <x:c r="C15" s="16" t="str">
+        <x:v>Use the specific relevant landing page and route readers to the right form, call action or shop page. Future article permalinks must be checked after publication.</x:v>
+      </x:c>
+      <x:c r="D15" s="16" t="str">
+        <x:v>Public phone numbers differ from the campaign number in some views; confirm number roles and tracking before edits.</x:v>
+      </x:c>
+      <x:c r="E15" s="16" t="str">
+        <x:v>Route check</x:v>
+      </x:c>
+      <x:c r="F15" s="16" t="str">
+        <x:v>https://aladdincleans.com/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4302,7 +4402,7 @@
         <x:v>Relevant existing customers or subscribers, if a suitable segment exists. Check Constant Contact schedule and suppress duplicates before sending.</x:v>
       </x:c>
       <x:c r="D6" s="30" t="str">
-        <x:v>October 29 Oriental rug evaluation guide, exact live permalink</x:v>
+        <x:v>Oct 29 rug evaluation guide: exact URL after publication → verified residential request form or call action</x:v>
       </x:c>
       <x:c r="E6" s="30" t="str">
         <x:v>Use a recognizable person + Aladdin sender, a specific subject and conversational plain text with no logo/header. Answer one rug-care question; link to the guide and its verified contact action.</x:v>
@@ -4325,7 +4425,7 @@
         <x:v>Conditional: review first email relevance, clicks, tagged visits, inquiries and unsubscribes; check existing sends and availability before proceeding.</x:v>
       </x:c>
       <x:c r="D7" s="30" t="str">
-        <x:v>November 19 practical pre-guest care guide, exact live permalink</x:v>
+        <x:v>Nov 19 pre-guest guide: exact URL after publication → verified residential request form or call action</x:v>
       </x:c>
       <x:c r="E7" s="30" t="str">
         <x:v>Use the same person + company, specific subject and plain-text approach. Offer a useful planning answer without holiday urgency or unverified availability.</x:v>
@@ -4380,7 +4480,7 @@
         <x:v>Post/email ID, tagged URL, article or service landing page, CTA and final contact path</x:v>
       </x:c>
       <x:c r="C11" s="30" t="str">
-        <x:v>Facebook links to the exact matching Aladdin page; email links to the hub; Instagram caption uses 210-361-3930, without a raw URL.</x:v>
+        <x:v>Facebook links to the exact matching Aladdin page; email links to its hub guide; Instagram caption uses approved phone CTA, with no raw URL. Confirm the channel number before scheduling.</x:v>
       </x:c>
       <x:c r="D11" s="17"/>
       <x:c r="E11" s="17"/>
@@ -4395,7 +4495,7 @@
         <x:v>Tagged sessions to each hub and contact path; form events; phone events</x:v>
       </x:c>
       <x:c r="C12" s="30" t="str">
-        <x:v>Verify event definitions after the Oct 19 tracking changes. Count forms and phone actions separately; inspect source and service fit.</x:v>
+        <x:v>Email drafts are in the Email Drafts tab. Oct 30 rug-care and Nov 20 pre-guest sends are segmented plans, not sent campaigns. Keep frequency low while unsubscribes are elevated.</x:v>
       </x:c>
       <x:c r="D12" s="17"/>
       <x:c r="E12" s="17"/>
@@ -4484,4 +4584,1463 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="88" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="32" t="str">
+        <x:v>Post to website to inquiry path map</x:v>
+      </x:c>
+      <x:c r="B2" s="32"/>
+      <x:c r="C2" s="32"/>
+      <x:c r="D2" s="32"/>
+      <x:c r="E2" s="32"/>
+      <x:c r="F2" s="32"/>
+      <x:c r="G2" s="32"/>
+    </x:row>
+    <x:row r="3" ht="38" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Each row shows the intended reader route. Scheduled posts still need their saved CoSchedule links checked; unpublished article permalinks cannot be verified yet.</x:v>
+      </x:c>
+      <x:c r="B3" s="16"/>
+      <x:c r="C3" s="16"/>
+      <x:c r="D3" s="16"/>
+      <x:c r="E3" s="16"/>
+      <x:c r="F3" s="16"/>
+      <x:c r="G3" s="16"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="37" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B5" s="37" t="str">
+        <x:v>Post or editorial assignment</x:v>
+      </x:c>
+      <x:c r="C5" s="37" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="D5" s="37" t="str">
+        <x:v>Website entry destination</x:v>
+      </x:c>
+      <x:c r="E5" s="37" t="str">
+        <x:v>Final next action</x:v>
+      </x:c>
+      <x:c r="F5" s="37" t="str">
+        <x:v>Before scheduling or audit</x:v>
+      </x:c>
+      <x:c r="G5" s="37" t="str">
+        <x:v>Measure</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>A spill on a valuable rug: first response</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D6" s="30" t="str">
+        <x:v>https://aladdincleans.com/blog/oriental-rugs/what-to-do-first-after-a-spill-on-a-rug/</x:v>
+      </x:c>
+      <x:c r="E6" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F6" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G6" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="70" customHeight="1">
+      <x:c r="A7" s="30" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>Plan around traffic and access</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D7" s="30" t="str">
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
+      </x:c>
+      <x:c r="E7" s="30" t="str">
+        <x:v>Commercial page contact action or call; confirm current number and routing</x:v>
+      </x:c>
+      <x:c r="F7" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G7" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="70" customHeight="1">
+      <x:c r="A8" s="30" t="str">
+        <x:v>2026-10-17</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>What home-care question should we answer next?</x:v>
+      </x:c>
+      <x:c r="C8" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E8" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F8" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Instagram caption and phone action; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G8" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="70" customHeight="1">
+      <x:c r="A9" s="30" t="str">
+        <x:v>2026-10-18</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>Listen and record questions</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D9" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E9" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F9" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G9" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="70" customHeight="1">
+      <x:c r="A10" s="30" t="str">
+        <x:v>2026-10-19</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>What a clear care plan should tell you</x:v>
+      </x:c>
+      <x:c r="C10" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E10" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F10" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G10" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="70" customHeight="1">
+      <x:c r="A11" s="30" t="str">
+        <x:v>2026-10-20</x:v>
+      </x:c>
+      <x:c r="B11" s="30" t="str">
+        <x:v>The first walkthrough, step by step</x:v>
+      </x:c>
+      <x:c r="C11" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D11" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E11" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F11" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G11" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="70" customHeight="1">
+      <x:c r="A12" s="30" t="str">
+        <x:v>2026-10-21</x:v>
+      </x:c>
+      <x:c r="B12" s="30" t="str">
+        <x:v>What would help you feel prepared for a service visit?</x:v>
+      </x:c>
+      <x:c r="C12" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D12" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E12" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F12" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="70" customHeight="1">
+      <x:c r="A13" s="30" t="str">
+        <x:v>2026-10-22</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>What a clear estimate should explain</x:v>
+      </x:c>
+      <x:c r="C13" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D13" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E13" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="70" customHeight="1">
+      <x:c r="A14" s="30" t="str">
+        <x:v>2026-10-23</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>Respect for the home begins with questions</x:v>
+      </x:c>
+      <x:c r="C14" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D14" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E14" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F14" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G14" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="70" customHeight="1">
+      <x:c r="A15" s="30" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>Which part of a visit deserves a clearer explanation?</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>Scheduled</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E15" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F15" s="30" t="str">
+        <x:v>Scheduled in CoSchedule: verify the actual saved Facebook destination and Instagram phone CTA; do not treat this plan as proof of the live post.</x:v>
+      </x:c>
+      <x:c r="G15" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="30" t="str">
+        <x:v>2026-10-25</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>Listen and refine</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E16" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F16" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G16" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="70" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>2026-10-26</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>When is a rug worth a closer evaluation?</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
+      </x:c>
+      <x:c r="E17" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F17" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G17" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="70" customHeight="1">
+      <x:c r="A18" s="30" t="str">
+        <x:v>2026-10-27</x:v>
+      </x:c>
+      <x:c r="B18" s="30" t="str">
+        <x:v>What an intake can reveal</x:v>
+      </x:c>
+      <x:c r="C18" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D18" s="30" t="str">
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
+      </x:c>
+      <x:c r="E18" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F18" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G18" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="70" customHeight="1">
+      <x:c r="A19" s="30" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c r="B19" s="30" t="str">
+        <x:v>What do you know about your rug?</x:v>
+      </x:c>
+      <x:c r="C19" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D19" s="30" t="str">
+        <x:v>https://aladdincleans.com/oriental-rugs/rug-cleaning/</x:v>
+      </x:c>
+      <x:c r="E19" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F19" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G19" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="70" customHeight="1">
+      <x:c r="A20" s="30" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>What an Oriental rug evaluation should cover</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="str">
+        <x:v>Oct 29 rug evaluation guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E20" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F20" s="30" t="str">
+        <x:v>Publish Oct 29 rug evaluation guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G20" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="70" customHeight="1">
+      <x:c r="A21" s="30" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>Choosing a rug is personal</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>https://aladdincleans.com/rug-store/</x:v>
+      </x:c>
+      <x:c r="E21" s="30" t="str">
+        <x:v>Shop/gallery or current product page; verify stock and price</x:v>
+      </x:c>
+      <x:c r="F21" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag. Recheck inventory and price.</x:v>
+      </x:c>
+      <x:c r="G21" s="30" t="str">
+        <x:v>Tagged gallery or product visits and shopping actions; keep this distinct from cleaning inquiries</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="70" customHeight="1">
+      <x:c r="A22" s="30" t="str">
+        <x:v>2026-10-31</x:v>
+      </x:c>
+      <x:c r="B22" s="30" t="str">
+        <x:v>After the rug evaluation guide, what would you ask next?</x:v>
+      </x:c>
+      <x:c r="C22" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D22" s="30" t="str">
+        <x:v>Oct 29 rug evaluation guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E22" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F22" s="30" t="str">
+        <x:v>Publish Oct 29 rug evaluation guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G22" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="70" customHeight="1">
+      <x:c r="A23" s="30" t="str">
+        <x:v>2026-11-01</x:v>
+      </x:c>
+      <x:c r="B23" s="30" t="str">
+        <x:v>Listen and update FAQ</x:v>
+      </x:c>
+      <x:c r="C23" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D23" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E23" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F23" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G23" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="70" customHeight="1">
+      <x:c r="A24" s="30" t="str">
+        <x:v>2026-11-02</x:v>
+      </x:c>
+      <x:c r="B24" s="30" t="str">
+        <x:v>Three questions before upholstery care</x:v>
+      </x:c>
+      <x:c r="C24" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D24" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
+      </x:c>
+      <x:c r="E24" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F24" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G24" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="70" customHeight="1">
+      <x:c r="A25" s="30" t="str">
+        <x:v>2026-11-03</x:v>
+      </x:c>
+      <x:c r="B25" s="30" t="str">
+        <x:v>How a fabric question becomes a care plan</x:v>
+      </x:c>
+      <x:c r="C25" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D25" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
+      </x:c>
+      <x:c r="E25" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F25" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G25" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="70" customHeight="1">
+      <x:c r="A26" s="30" t="str">
+        <x:v>2026-11-04</x:v>
+      </x:c>
+      <x:c r="B26" s="30" t="str">
+        <x:v>Which surface do you have a question about?</x:v>
+      </x:c>
+      <x:c r="C26" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D26" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
+      </x:c>
+      <x:c r="E26" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F26" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G26" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="70" customHeight="1">
+      <x:c r="A27" s="30" t="str">
+        <x:v>2026-11-05</x:v>
+      </x:c>
+      <x:c r="B27" s="30" t="str">
+        <x:v>A practical upholstery care conversation</x:v>
+      </x:c>
+      <x:c r="C27" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D27" s="30" t="str">
+        <x:v>Nov 5 upholstery guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E27" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F27" s="30" t="str">
+        <x:v>Publish Nov 5 upholstery guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G27" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="70" customHeight="1">
+      <x:c r="A28" s="30" t="str">
+        <x:v>2026-11-06</x:v>
+      </x:c>
+      <x:c r="B28" s="30" t="str">
+        <x:v>Why careful recommendations matter</x:v>
+      </x:c>
+      <x:c r="C28" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D28" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/upholstery-cleaning/</x:v>
+      </x:c>
+      <x:c r="E28" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F28" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G28" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="70" customHeight="1">
+      <x:c r="A29" s="30" t="str">
+        <x:v>2026-11-07</x:v>
+      </x:c>
+      <x:c r="B29" s="30" t="str">
+        <x:v>What would you ask about a favorite chair?</x:v>
+      </x:c>
+      <x:c r="C29" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D29" s="30" t="str">
+        <x:v>Nov 5 upholstery guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E29" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F29" s="30" t="str">
+        <x:v>Publish Nov 5 upholstery guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G29" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="70" customHeight="1">
+      <x:c r="A30" s="30" t="str">
+        <x:v>2026-11-08</x:v>
+      </x:c>
+      <x:c r="B30" s="30" t="str">
+        <x:v>Listen and log needs</x:v>
+      </x:c>
+      <x:c r="C30" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D30" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E30" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F30" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G30" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="70" customHeight="1">
+      <x:c r="A31" s="30" t="str">
+        <x:v>2026-11-09</x:v>
+      </x:c>
+      <x:c r="B31" s="30" t="str">
+        <x:v>What to know before water affects a room</x:v>
+      </x:c>
+      <x:c r="C31" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D31" s="30" t="str">
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
+      </x:c>
+      <x:c r="E31" s="30" t="str">
+        <x:v>Call for an active issue from water-damage page; confirm current emergency number</x:v>
+      </x:c>
+      <x:c r="F31" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag. Operations must approve safety and response language.</x:v>
+      </x:c>
+      <x:c r="G31" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="70" customHeight="1">
+      <x:c r="A32" s="30" t="str">
+        <x:v>2026-11-10</x:v>
+      </x:c>
+      <x:c r="B32" s="30" t="str">
+        <x:v>What a useful incident record includes</x:v>
+      </x:c>
+      <x:c r="C32" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D32" s="30" t="str">
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
+      </x:c>
+      <x:c r="E32" s="30" t="str">
+        <x:v>Call for an active issue from water-damage page; confirm current emergency number</x:v>
+      </x:c>
+      <x:c r="F32" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag. Operations must approve safety and response language.</x:v>
+      </x:c>
+      <x:c r="G32" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="70" customHeight="1">
+      <x:c r="A33" s="30" t="str">
+        <x:v>2026-11-11</x:v>
+      </x:c>
+      <x:c r="B33" s="30" t="str">
+        <x:v>What should you document after water enters a room?</x:v>
+      </x:c>
+      <x:c r="C33" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D33" s="30" t="str">
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
+      </x:c>
+      <x:c r="E33" s="30" t="str">
+        <x:v>Call for an active issue from water-damage page; confirm current emergency number</x:v>
+      </x:c>
+      <x:c r="F33" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag. Operations must approve safety and response language.</x:v>
+      </x:c>
+      <x:c r="G33" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="70" customHeight="1">
+      <x:c r="A34" s="30" t="str">
+        <x:v>2026-11-12</x:v>
+      </x:c>
+      <x:c r="B34" s="30" t="str">
+        <x:v>What a clear water-damage response should explain</x:v>
+      </x:c>
+      <x:c r="C34" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D34" s="30" t="str">
+        <x:v>Nov 12 water response guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E34" s="30" t="str">
+        <x:v>Call for an active issue from water-damage page; confirm current emergency number</x:v>
+      </x:c>
+      <x:c r="F34" s="30" t="str">
+        <x:v>Publish Nov 12 water response guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA. Operations must approve safety and response language.</x:v>
+      </x:c>
+      <x:c r="G34" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="70" customHeight="1">
+      <x:c r="A35" s="30" t="str">
+        <x:v>2026-11-13</x:v>
+      </x:c>
+      <x:c r="B35" s="30" t="str">
+        <x:v>The people behind a calm response</x:v>
+      </x:c>
+      <x:c r="C35" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D35" s="30" t="str">
+        <x:v>https://aladdincleans.com/water-damage-restoration/</x:v>
+      </x:c>
+      <x:c r="E35" s="30" t="str">
+        <x:v>Call for an active issue from water-damage page; confirm current emergency number</x:v>
+      </x:c>
+      <x:c r="F35" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag. Operations must approve safety and response language.</x:v>
+      </x:c>
+      <x:c r="G35" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="70" customHeight="1">
+      <x:c r="A36" s="30" t="str">
+        <x:v>2026-11-14</x:v>
+      </x:c>
+      <x:c r="B36" s="30" t="str">
+        <x:v>Who has the first call and site access?</x:v>
+      </x:c>
+      <x:c r="C36" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D36" s="30" t="str">
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
+      </x:c>
+      <x:c r="E36" s="30" t="str">
+        <x:v>Commercial page contact action or call; confirm current number and routing</x:v>
+      </x:c>
+      <x:c r="F36" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G36" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="70" customHeight="1">
+      <x:c r="A37" s="30" t="str">
+        <x:v>2026-11-15</x:v>
+      </x:c>
+      <x:c r="B37" s="30" t="str">
+        <x:v>Listen and review readiness questions</x:v>
+      </x:c>
+      <x:c r="C37" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D37" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E37" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F37" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G37" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="70" customHeight="1">
+      <x:c r="A38" s="30" t="str">
+        <x:v>2026-11-16</x:v>
+      </x:c>
+      <x:c r="B38" s="30" t="str">
+        <x:v>Plan the spaces that matter before guests arrive</x:v>
+      </x:c>
+      <x:c r="C38" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D38" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E38" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F38" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G38" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="70" customHeight="1">
+      <x:c r="A39" s="30" t="str">
+        <x:v>2026-11-17</x:v>
+      </x:c>
+      <x:c r="B39" s="30" t="str">
+        <x:v>How to prepare for a service visit</x:v>
+      </x:c>
+      <x:c r="C39" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D39" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E39" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F39" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G39" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="70" customHeight="1">
+      <x:c r="A40" s="30" t="str">
+        <x:v>2026-11-18</x:v>
+      </x:c>
+      <x:c r="B40" s="30" t="str">
+        <x:v>Which room matters most when people gather?</x:v>
+      </x:c>
+      <x:c r="C40" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D40" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E40" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F40" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G40" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="70" customHeight="1">
+      <x:c r="A41" s="30" t="str">
+        <x:v>2026-11-19</x:v>
+      </x:c>
+      <x:c r="B41" s="30" t="str">
+        <x:v>A calm pre-guest property-care plan</x:v>
+      </x:c>
+      <x:c r="C41" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D41" s="30" t="str">
+        <x:v>Nov 19 pre-guest guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E41" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F41" s="30" t="str">
+        <x:v>Publish Nov 19 pre-guest guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G41" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="70" customHeight="1">
+      <x:c r="A42" s="30" t="str">
+        <x:v>2026-11-20</x:v>
+      </x:c>
+      <x:c r="B42" s="30" t="str">
+        <x:v>Clear communication makes planning easier</x:v>
+      </x:c>
+      <x:c r="C42" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D42" s="30" t="str">
+        <x:v>https://aladdincleans.com/residential-services/</x:v>
+      </x:c>
+      <x:c r="E42" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F42" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G42" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="70" customHeight="1">
+      <x:c r="A43" s="30" t="str">
+        <x:v>2026-11-21</x:v>
+      </x:c>
+      <x:c r="B43" s="30" t="str">
+        <x:v>What is your last planning question?</x:v>
+      </x:c>
+      <x:c r="C43" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D43" s="30" t="str">
+        <x:v>Nov 19 pre-guest guide: exact URL pending publication</x:v>
+      </x:c>
+      <x:c r="E43" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F43" s="30" t="str">
+        <x:v>Publish Nov 19 pre-guest guide, verify its live permalink and relevant CTA, then insert that URL in Facebook/email before scheduling. Keep Instagram phone CTA.</x:v>
+      </x:c>
+      <x:c r="G43" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="70" customHeight="1">
+      <x:c r="A44" s="30" t="str">
+        <x:v>2026-11-22</x:v>
+      </x:c>
+      <x:c r="B44" s="30" t="str">
+        <x:v>Listen before the holiday week</x:v>
+      </x:c>
+      <x:c r="C44" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D44" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E44" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F44" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G44" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="70" customHeight="1">
+      <x:c r="A45" s="30" t="str">
+        <x:v>2026-11-23</x:v>
+      </x:c>
+      <x:c r="B45" s="30" t="str">
+        <x:v>Before a holiday closure, confirm the basics</x:v>
+      </x:c>
+      <x:c r="C45" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D45" s="30" t="str">
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
+      </x:c>
+      <x:c r="E45" s="30" t="str">
+        <x:v>Commercial page contact action or call; confirm current number and routing</x:v>
+      </x:c>
+      <x:c r="F45" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G45" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="70" customHeight="1">
+      <x:c r="A46" s="30" t="str">
+        <x:v>2026-11-24</x:v>
+      </x:c>
+      <x:c r="B46" s="30" t="str">
+        <x:v>A practical surface-care walkthrough</x:v>
+      </x:c>
+      <x:c r="C46" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D46" s="30" t="str">
+        <x:v>https://aladdincleans.com/commercial-services/</x:v>
+      </x:c>
+      <x:c r="E46" s="30" t="str">
+        <x:v>Commercial page contact action or call; confirm current number and routing</x:v>
+      </x:c>
+      <x:c r="F46" s="30" t="str">
+        <x:v>Verify the exact Facebook URL; Instagram has no raw caption URL. Confirm matching page CTA, contact route and tracking tag.</x:v>
+      </x:c>
+      <x:c r="G46" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="70" customHeight="1">
+      <x:c r="A47" s="30" t="str">
+        <x:v>2026-11-25</x:v>
+      </x:c>
+      <x:c r="B47" s="30" t="str">
+        <x:v>A local thank-you, grounded in people</x:v>
+      </x:c>
+      <x:c r="C47" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D47" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E47" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F47" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G47" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="70" customHeight="1">
+      <x:c r="A48" s="30" t="str">
+        <x:v>2026-11-26</x:v>
+      </x:c>
+      <x:c r="B48" s="30" t="str">
+        <x:v>Thanksgiving listening only</x:v>
+      </x:c>
+      <x:c r="C48" s="30" t="str">
+        <x:v>Listen</x:v>
+      </x:c>
+      <x:c r="D48" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E48" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F48" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G48" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="70" customHeight="1">
+      <x:c r="A49" s="30" t="str">
+        <x:v>2026-11-27</x:v>
+      </x:c>
+      <x:c r="B49" s="30" t="str">
+        <x:v>After a gathering, respond to a rug spill calmly</x:v>
+      </x:c>
+      <x:c r="C49" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D49" s="30" t="str">
+        <x:v>https://aladdincleans.com/blog/oriental-rugs/what-to-do-first-after-a-spill-on-a-rug/</x:v>
+      </x:c>
+      <x:c r="E49" s="30" t="str">
+        <x:v>https://aladdincleans.com/locations/schedule-online/</x:v>
+      </x:c>
+      <x:c r="F49" s="30" t="str">
+        <x:v>Recheck the existing guide and its current CTA before scheduling the November 27 post.</x:v>
+      </x:c>
+      <x:c r="G49" s="30" t="str">
+        <x:v>Tagged entry sessions; separate form and phone events; qualified inquiries where applicable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="70" customHeight="1">
+      <x:c r="A50" s="30" t="str">
+        <x:v>2026-11-28</x:v>
+      </x:c>
+      <x:c r="B50" s="30" t="str">
+        <x:v>What should we explain in December?</x:v>
+      </x:c>
+      <x:c r="C50" s="30" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="D50" s="30" t="str">
+        <x:v>No website link planned</x:v>
+      </x:c>
+      <x:c r="E50" s="30" t="str">
+        <x:v>Reply, listen or collect topic questions</x:v>
+      </x:c>
+      <x:c r="F50" s="30" t="str">
+        <x:v>Do not invent a website path for a listening day or a platform-only prompt.</x:v>
+      </x:c>
+      <x:c r="G50" s="30" t="str">
+        <x:v>Useful questions or replies; feed into the next content review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="52" customHeight="1">
+      <x:c r="A52" s="38" t="str">
+        <x:v>Channel rule</x:v>
+      </x:c>
+      <x:c r="B52" s="16" t="str">
+        <x:v>Facebook and email link to the exact relevant Aladdin page with a campaign tag. Instagram caption uses the campaign phone CTA; verify the approved number and call tracking before scheduling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="52" customHeight="1">
+      <x:c r="A53" s="38" t="str">
+        <x:v>Contact rule</x:v>
+      </x:c>
+      <x:c r="B53" s="16" t="str">
+        <x:v>Residential and rug-care content can lead to the residential request form. Commercial and active water-damage content need their own confirmed contact or call path. Shopping posts lead to gallery or product pages.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="52" customHeight="1">
+      <x:c r="A54" s="38" t="str">
+        <x:v>Number check</x:v>
+      </x:c>
+      <x:c r="B54" s="16" t="str">
+        <x:v>The calendar names 210-361-3930 for Instagram, while the public site can show a different phone number. Confirm which tracked number belongs to each channel and to emergency calls before changing captions.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A3:G3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="65" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="64" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="65" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="61" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="40" t="str">
+        <x:v>Connected content: social, blog, email and inquiry</x:v>
+      </x:c>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+      <x:c r="F2" s="40"/>
+    </x:row>
+    <x:row r="3" ht="35" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Use these briefs with the 45-Day Calendar and Post Path Map. These are production instructions and draft copy, not proof of publication or measured lift.</x:v>
+      </x:c>
+      <x:c r="B3" s="16"/>
+      <x:c r="C3" s="16"/>
+      <x:c r="D3" s="16"/>
+      <x:c r="E3" s="16"/>
+      <x:c r="F3" s="16"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>Sequence / publish gate</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>Useful social promise</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>Blog or page handoff</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>Email / return loop</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>Action and conversion route</x:v>
+      </x:c>
+      <x:c r="F5" s="45" t="str">
+        <x:v>Evidence and approval gate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="120" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>Rug care · Oct 26–31</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>Help owners recognize what is worth asking before specialty cleaning; show the real intake process and invite a specific rug question.</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>Oct 29 evaluation guide answers history, construction, condition, dye and repair questions; FB links exact article after publication. Oct 30 gallery post is a separate shopping path.</x:v>
+      </x:c>
+      <x:c r="D6" s="30" t="str">
+        <x:v>Oct 30 segmented email: owners who have shown interest in rug care; one helpful assessment question plus article link. Exclude non-relevant recipients where possible.</x:v>
+      </x:c>
+      <x:c r="E6" s="30" t="str">
+        <x:v>Guide → rug-care inquiry via improved residential form or approved phone action. Gallery → product page/shopping; measure separately.</x:v>
+      </x:c>
+      <x:c r="F6" s="30" t="str">
+        <x:v>Use actual Aladdin rug and process photos. Verify article link, form route, gallery inventory and product prices.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="120" customHeight="1">
+      <x:c r="A7" s="30" t="str">
+        <x:v>Upholstery · Nov 2–7</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>Ask what fabric, condition and outcome the owner cares about; show how those answers shape a conversation.</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>Nov 5 owner guide covers material, condition, expectations, timing and aftercare; FB links exact guide after publication.</x:v>
+      </x:c>
+      <x:c r="D7" s="30" t="str">
+        <x:v>Optional: use a short guide excerpt only if segment is relevant and frequency permits; no extra blast while unsubscribes are elevated.</x:v>
+      </x:c>
+      <x:c r="E7" s="30" t="str">
+        <x:v>Guide → improved residential form with Upholstery or Not sure selected, or approved phone action.</x:v>
+      </x:c>
+      <x:c r="F7" s="30" t="str">
+        <x:v>No universal method or guaranteed result. Obtain approval for customer/process example and real photo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="120" customHeight="1">
+      <x:c r="A8" s="30" t="str">
+        <x:v>Water response · Nov 9–14</x:v>
+      </x:c>
+      <x:c r="B8" s="30" t="str">
+        <x:v>Give safe, useful documentation and contact-prep questions. Separate active-issue action from educational reading.</x:v>
+      </x:c>
+      <x:c r="C8" s="30" t="str">
+        <x:v>Nov 12 operations-reviewed guide provides safe first-step and initial-conversation context; FB links it after publication.</x:v>
+      </x:c>
+      <x:c r="D8" s="30" t="str">
+        <x:v>Use only a relevant educational segment and approved cadence. For active issues, show the confirmed call route first.</x:v>
+      </x:c>
+      <x:c r="E8" s="30" t="str">
+        <x:v>Active issue → verified restoration phone action. Educational reader → guide and commercial/residential follow-up as applicable.</x:v>
+      </x:c>
+      <x:c r="F8" s="30" t="str">
+        <x:v>Operations approves safety wording, availability language and correct active-issue phone number.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="120" customHeight="1">
+      <x:c r="A9" s="30" t="str">
+        <x:v>Pre-guest care · Nov 16–21</x:v>
+      </x:c>
+      <x:c r="B9" s="30" t="str">
+        <x:v>Help residents prioritize spaces, material concerns and realistic timing; show what to share before a visit.</x:v>
+      </x:c>
+      <x:c r="C9" s="30" t="str">
+        <x:v>Nov 19 planning guide gives checklist and direct handoff to the improved residential request form.</x:v>
+      </x:c>
+      <x:c r="D9" s="30" t="str">
+        <x:v>Nov 20 segmented email: deliver checklist and link to guide; a second, light follow-up only for interested readers and if frequency allows.</x:v>
+      </x:c>
+      <x:c r="E9" s="30" t="str">
+        <x:v>Guide → improved form (service choice, Not sure option, Special Requests) or approved phone; track form and call events separately.</x:v>
+      </x:c>
+      <x:c r="F9" s="30" t="str">
+        <x:v>No urgency, availability or outcome promise. Verify actual form choices and email automation before sending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="120" customHeight="1">
+      <x:c r="A10" s="30" t="str">
+        <x:v>Holiday/commercial · Nov 23–28</x:v>
+      </x:c>
+      <x:c r="B10" s="30" t="str">
+        <x:v>Offer facility closure checklist, a real walkthrough and a helpful rug-spill guide reuse; avoid holiday sales pressure.</x:v>
+      </x:c>
+      <x:c r="C10" s="30" t="str">
+        <x:v>Commercial service page for Nov 23–24; existing rug-spill article for Nov 27.</x:v>
+      </x:c>
+      <x:c r="D10" s="30" t="str">
+        <x:v>No general holiday blast planned. Use replies and tagged guide visits to shape December topics.</x:v>
+      </x:c>
+      <x:c r="E10" s="30" t="str">
+        <x:v>Commercial → commercial contact/call. Rug spill → article then residential inquiry/phone.</x:v>
+      </x:c>
+      <x:c r="F10" s="30" t="str">
+        <x:v>Verify hours, service contact route and any holiday operation detail before publishing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="46" t="str">
+        <x:v>Channel copy examples: edit against the final article and approved number before scheduling</x:v>
+      </x:c>
+      <x:c r="B12" s="46"/>
+      <x:c r="C12" s="46"/>
+      <x:c r="D12" s="46"/>
+      <x:c r="E12" s="46"/>
+      <x:c r="F12" s="46"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="45" t="str">
+        <x:v>Campaign</x:v>
+      </x:c>
+      <x:c r="B13" s="45" t="str">
+        <x:v>Facebook draft (add exact verified article URL)</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>Instagram draft (no raw URL; add approved phone)</x:v>
+      </x:c>
+      <x:c r="D13" s="45" t="str">
+        <x:v>Production note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="160" customHeight="1">
+      <x:c r="A14" s="30" t="str">
+        <x:v>Rug evaluation · Oct 29</x:v>
+      </x:c>
+      <x:c r="B14" s="30" t="str">
+        <x:v>Before an Oriental rug is cleaned, what should be checked? Its construction, dyes, condition and prior repairs can all shape the conversation. Our new guide walks through the questions to ask before a care plan is recommended. Read it here: [verified Oct 29 article URL]. Have a rug question? The guide shows how to reach Aladdin.</x:v>
+      </x:c>
+      <x:c r="C14" s="30" t="str">
+        <x:v>A beautiful rug can have a history you cannot see in one photo. Ask what is known about its fiber, dyes, condition and past repairs before deciding on care. Our evaluation guide covers the conversation. Call Aladdin at 210-361-3930 with your rug question.</x:v>
+      </x:c>
+      <x:c r="D14" s="30" t="str">
+        <x:v>Use actual rug and intake photography. Number requires channel confirmation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="160" customHeight="1">
+      <x:c r="A15" s="30" t="str">
+        <x:v>Upholstery · Nov 5</x:v>
+      </x:c>
+      <x:c r="B15" s="30" t="str">
+        <x:v>That favorite chair has a fabric, a history and a job in your home. Before care begins, ask what the material is, what has changed and what a realistic result may look like. Our new upholstery guide helps you prepare: [verified Nov 5 article URL]. You can reach Aladdin from the guide.</x:v>
+      </x:c>
+      <x:c r="C15" s="30" t="str">
+        <x:v>Before upholstery care, ask three things: What is the fabric? What has changed? What result matters to you? A useful first conversation starts there. Call Aladdin at 210-361-3930 to talk through your furniture.</x:v>
+      </x:c>
+      <x:c r="D15" s="30" t="str">
+        <x:v>Use approved furniture and team photos; avoid before/after promises.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="160" customHeight="1">
+      <x:c r="A16" s="30" t="str">
+        <x:v>Water response · Nov 12</x:v>
+      </x:c>
+      <x:c r="B16" s="30" t="str">
+        <x:v>When water affects a room, the first conversation is easier when you know what happened, what you can document safely and who can give access. Our guide explains those questions and the limits of an initial assessment: [verified Nov 12 article URL]. For an active issue, use the confirmed call action on the page.</x:v>
+      </x:c>
+      <x:c r="C16" s="30" t="str">
+        <x:v>If water affects a room, start with safety. From a safe place, note when you noticed it, where it is and who can give access. For an active issue, call Aladdin at [confirmed active-issue number].</x:v>
+      </x:c>
+      <x:c r="D16" s="30" t="str">
+        <x:v>Operations must approve safety guidance and number before scheduling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="160" customHeight="1">
+      <x:c r="A17" s="30" t="str">
+        <x:v>Pre-guest planning · Nov 19</x:v>
+      </x:c>
+      <x:c r="B17" s="30" t="str">
+        <x:v>Getting a home ready for guests starts with priorities: the spaces people will use, the materials that need special attention and the time available. Our planning guide gives you a simple checklist and a way to share your needs with Aladdin: [verified Nov 19 article URL].</x:v>
+      </x:c>
+      <x:c r="C17" s="30" t="str">
+        <x:v>Before guests arrive, make a short list: high-use spaces, delicate materials and your ideal timing. Need help deciding which service fits? You can explain that when you contact Aladdin. Call 210-361-3930 with your home-care question.</x:v>
+      </x:c>
+      <x:c r="D17" s="30" t="str">
+        <x:v>Use genuine home/team photography; do not imply guaranteed appointment availability.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A3:F3"/>
+    <x:mergeCell ref="A12:F12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="90" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="70" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2">
+      <x:c r="A2" s="40" t="str">
+        <x:v>Segmented email drafts tied to the guides</x:v>
+      </x:c>
+      <x:c r="B2" s="40"/>
+      <x:c r="C2" s="40"/>
+      <x:c r="D2" s="40"/>
+      <x:c r="E2" s="40"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="16" t="str">
+        <x:v>Drafts need final article URLs, list segmentation, approval and a live send test. Neither is marked as sent.</x:v>
+      </x:c>
+      <x:c r="B3" s="16"/>
+      <x:c r="C3" s="16"/>
+      <x:c r="D3" s="16"/>
+      <x:c r="E3" s="16"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="45" t="str">
+        <x:v>Target date and segment</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str">
+        <x:v>Subject / preview</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="str">
+        <x:v>Email body draft</x:v>
+      </x:c>
+      <x:c r="D5" s="45" t="str">
+        <x:v>Primary button and landing</x:v>
+      </x:c>
+      <x:c r="E5" s="45" t="str">
+        <x:v>Follow-up / measurement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="178" customHeight="1">
+      <x:c r="A6" s="30" t="str">
+        <x:v>Oct 30 · rug-care interested contacts</x:v>
+      </x:c>
+      <x:c r="B6" s="30" t="str">
+        <x:v>Subject: Before you decide how to care for a rug
+Preview: Five questions to bring to the conversation.</x:v>
+      </x:c>
+      <x:c r="C6" s="30" t="str">
+        <x:v>A rug can carry years of use, repair and meaning. A useful first question is: what do we know about its construction, condition and past care? We put together a short guide to help you ask the right questions before a cleaning plan is recommended. [Button: Read the rug evaluation guide] If you would like Aladdin to look at your rug, the guide shows you how to describe it and start a conversation.</x:v>
+      </x:c>
+      <x:c r="D6" s="30" t="str">
+        <x:v>Read the rug evaluation guide → verified Oct 29 article URL → rug-care inquiry form or approved call action</x:v>
+      </x:c>
+      <x:c r="E6" s="30" t="str">
+        <x:v>Track delivered, human opens where reliable, unique clicks, tagged guide visits, form and phone events separately, qualified inquiry notes. Suppress recent unsubscribers; no second send unless useful.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="178" customHeight="1">
+      <x:c r="A7" s="30" t="str">
+        <x:v>Nov 20 · residential contacts with pre-guest interest</x:v>
+      </x:c>
+      <x:c r="B7" s="30" t="str">
+        <x:v>Subject: A simpler plan for the spaces guests will use
+Preview: A short checklist before you request care.</x:v>
+      </x:c>
+      <x:c r="C7" s="30" t="str">
+        <x:v>Preparing for guests is easier when you decide what matters first. Note the rooms people will use, materials that need extra care and the time you have. Our short guide walks through those choices and what to share with Aladdin. [Button: Read the home-care planning guide] If you are unsure which service fits, the request form lets you explain your needs and ask for a conversation.</x:v>
+      </x:c>
+      <x:c r="D7" s="30" t="str">
+        <x:v>Read the pre-guest guide → verified Nov 19 article URL → improved residential request form or approved call action</x:v>
+      </x:c>
+      <x:c r="E7" s="30" t="str">
+        <x:v>Segment to relevant contacts and check frequency because unsubscribe rate rose. Track tagged guide visits, form and phone events, then review qualified inquiries.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>